<commit_message>
scan: seg0 2026-09-28 15:56 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq1_2026-09-24.xlsx
+++ b/output/full_scan/batch_seq1_2026-09-24.xlsx
@@ -555,7 +555,7 @@
         <v>76.76980525541725</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>31.41680151569321</v>
+        <v>31.4168015702786</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>1.008498413392119</v>
@@ -570,7 +570,7 @@
         <v>-1</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>24.49570838820415</v>
+        <v>24.49570838768908</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -605,10 +605,10 @@
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>79.89106156477303</v>
+        <v>79.89106143081827</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>53.06968872101748</v>
+        <v>53.06968890241327</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>2.741649652972179</v>
@@ -623,7 +623,7 @@
         <v>-1</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>1.590931852628519</v>
+        <v>1.590931853720629</v>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
@@ -658,10 +658,10 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>58.61440123410856</v>
+        <v>58.61440598226877</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>17.18896284450348</v>
+        <v>17.18896536541293</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>1.283795586748832</v>
@@ -676,7 +676,7 @@
         <v>-1</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>0.0340843764825968</v>
+        <v>0.0340843738862658</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
@@ -711,10 +711,10 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>56.55433796133729</v>
+        <v>56.55433808511896</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>40.34462201169195</v>
+        <v>40.34462239767203</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>0.1895911116324685</v>
@@ -729,7 +729,7 @@
         <v>-1</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>-0.07519359721979239</v>
+        <v>-0.0751935973454885</v>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
@@ -764,10 +764,10 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>60.93299628994088</v>
+        <v>60.93299614592757</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>26.89643561385643</v>
+        <v>26.89643566749574</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>0.999049460502734</v>
@@ -782,7 +782,7 @@
         <v>-1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>0.008277293785017001</v>
+        <v>0.0082772938571382</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
@@ -817,10 +817,10 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>58.09717153367886</v>
+        <v>58.09717154455284</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>23.99712451639491</v>
+        <v>23.99712473988518</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>0.7949632640336151</v>
@@ -835,7 +835,7 @@
         <v>-1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>-1.694069483020671</v>
+        <v>-1.694069483463693</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
@@ -870,10 +870,10 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>75.4911544196669</v>
+        <v>75.49115445273235</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>45.93921653948664</v>
+        <v>45.93921664763305</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>0.3006969482605902</v>
@@ -888,7 +888,7 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>0.068229957271102</v>
+        <v>0.06822995720925989</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
@@ -909,7 +909,7 @@
         <v/>
       </c>
       <c r="D9" s="2" t="n">
-        <v>678.8243237025708</v>
+        <v>678.8243237025711</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>25.45</v>
@@ -923,10 +923,10 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>65.72105385539237</v>
+        <v>65.72105379229193</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>37.09592352816865</v>
+        <v>37.09592363131511</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>0.7737003345632983</v>
@@ -941,7 +941,7 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>0.4556074238322736</v>
+        <v>0.4556074240692371</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
@@ -976,10 +976,10 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>68.29302356023521</v>
+        <v>68.29302357750073</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>48.45375435943801</v>
+        <v>48.45375427393484</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>0.1306458913668709</v>
@@ -1029,10 +1029,10 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>58.52601509604765</v>
+        <v>58.52601513452927</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>31.75787821900792</v>
+        <v>31.75787830596096</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>0.6525081178999347</v>
@@ -1082,10 +1082,10 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>60.71553075306982</v>
+        <v>60.71553072717938</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>34.27801528573151</v>
+        <v>34.27801534311887</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>0.4865206968699114</v>
@@ -1100,7 +1100,7 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>-0.3412781365943997</v>
+        <v>-0.341278136417837</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>60.28988304091983</v>
+        <v>60.28988319413902</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>18.1143949937001</v>
+        <v>18.11439463217432</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>1.438336874983999</v>
@@ -1153,7 +1153,7 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>0.0821446360632689</v>
+        <v>0.0821446363620538</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
@@ -1174,7 +1174,7 @@
         <v/>
       </c>
       <c r="D14" s="2" t="n">
-        <v>617.5477520375175</v>
+        <v>617.5477520375176</v>
       </c>
       <c r="E14" s="2" t="n">
         <v>12.5</v>
@@ -1188,10 +1188,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>53.53620395911947</v>
+        <v>53.53620403183438</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>21.43000304873751</v>
+        <v>21.43000327057417</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>0.7923255890524106</v>
@@ -1206,7 +1206,7 @@
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>0.001400774055535</v>
+        <v>0.001400773993717</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
@@ -1241,7 +1241,7 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>52.0899266163139</v>
+        <v>52.08992669373536</v>
       </c>
       <c r="I15" s="2" t="n">
         <v>10.26933187518033</v>
@@ -1294,10 +1294,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>51.63017679584309</v>
+        <v>51.63017684017526</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>28.26579655622348</v>
+        <v>28.26579695102428</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>0.5053244878320772</v>
@@ -1312,7 +1312,7 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>-0.6345949734404042</v>
+        <v>-0.6345949737597965</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
@@ -1347,10 +1347,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>71.14387127086208</v>
+        <v>71.14387143480535</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>36.11969021148665</v>
+        <v>36.11969027829939</v>
       </c>
       <c r="J17" s="2" t="n">
         <v>0.4134116033172695</v>
@@ -1365,7 +1365,7 @@
         <v>-1</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>0.1645810012960185</v>
+        <v>0.1645810011723649</v>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
@@ -1400,10 +1400,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>53.23083443494485</v>
+        <v>53.23083455005789</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>22.95163970565744</v>
+        <v>22.9516400415005</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>0.5460843204995706</v>
@@ -1418,7 +1418,7 @@
         <v>-1</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>-0.3531246927553171</v>
+        <v>-0.3531246933425762</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
@@ -1453,10 +1453,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>51.93921032324754</v>
+        <v>51.93921035606791</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>23.12381048549101</v>
+        <v>23.12381053684191</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>0.7842704691768611</v>
@@ -1471,7 +1471,7 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>0.002710323799178</v>
+        <v>0.0027103237888756</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
@@ -1506,10 +1506,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>44.40915745656954</v>
+        <v>44.40915747510478</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>15.14464571268223</v>
+        <v>15.14464573862796</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>0.2270158080671501</v>
@@ -1559,10 +1559,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>60.70055981570912</v>
+        <v>60.70055988039058</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>41.10032606681857</v>
+        <v>41.10032647486013</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>1.013911217114202</v>
@@ -1577,7 +1577,7 @@
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>0.07525803329222081</v>
+        <v>0.0752580332551296</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
@@ -1612,10 +1612,10 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>54.08287234028921</v>
+        <v>54.08287236493935</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>15.87081660312091</v>
+        <v>15.87081657321302</v>
       </c>
       <c r="J22" s="2" t="n">
         <v>0.407092049387347</v>
@@ -1630,7 +1630,7 @@
         <v>-1</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>-0.0417863745310384</v>
+        <v>-0.0417863745413435</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
@@ -1665,10 +1665,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>56.79220562504735</v>
+        <v>56.79220558377262</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>15.71171700071069</v>
+        <v>15.71171701028789</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>1.105566558177927</v>
@@ -1718,10 +1718,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>53.48114731366788</v>
+        <v>53.48114735305222</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>27.67049543656308</v>
+        <v>27.67049570260034</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>0.6537112824940586</v>
@@ -1736,7 +1736,7 @@
         <v>-1</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>-0.0210725773042343</v>
+        <v>-0.0210725773454489</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
@@ -1771,10 +1771,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>55.48243554290518</v>
+        <v>55.48243570517651</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>28.35361327067837</v>
+        <v>28.35361368408314</v>
       </c>
       <c r="J25" s="2" t="n">
         <v>0.6913980111746824</v>
@@ -1789,7 +1789,7 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>0.0247344407166157</v>
+        <v>0.0247344406259506</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
@@ -1810,7 +1810,7 @@
         <v/>
       </c>
       <c r="D26" s="2" t="n">
-        <v>496.2549857292478</v>
+        <v>496.2549857292479</v>
       </c>
       <c r="E26" s="2" t="n">
         <v>30.9</v>
@@ -1824,10 +1824,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>58.45887265302812</v>
+        <v>58.45887262375558</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>18.71366384816152</v>
+        <v>18.71366386828052</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>0.7051406157625537</v>
@@ -1842,7 +1842,7 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>0.2561221695572497</v>
+        <v>0.2561221695984589</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
@@ -1880,7 +1880,7 @@
         <v>48.82640971135586</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>12.27444449253986</v>
+        <v>12.2744445123444</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>1.531400252959722</v>
@@ -1930,10 +1930,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>49.68909414829141</v>
+        <v>49.6890941959791</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>21.08901584924069</v>
+        <v>21.08901632706459</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>0.7878205253041712</v>
@@ -1948,7 +1948,7 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>0.0164448750207527</v>
+        <v>0.0164448750413579</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
@@ -1986,7 +1986,7 @@
         <v>42.50966776336448</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>28.89237807896638</v>
+        <v>28.89237810026683</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>2.508345645706944</v>
@@ -2036,10 +2036,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>39.64992315276202</v>
+        <v>39.6499231005707</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>20.7979220757806</v>
+        <v>20.79792211131302</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>0.5862350659408259</v>
@@ -2054,7 +2054,7 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>0.0154544951585713</v>
+        <v>0.0154544952203942</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
@@ -2089,10 +2089,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46.10594759896849</v>
+        <v>46.10594747465212</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>17.46624579589394</v>
+        <v>17.46624585831511</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>0.4436552810998709</v>
@@ -2107,7 +2107,7 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>0.1259237989099998</v>
+        <v>0.1259237993221172</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
@@ -2128,7 +2128,7 @@
         <v/>
       </c>
       <c r="D32" s="2" t="n">
-        <v>462.555327862438</v>
+        <v>462.5553278624379</v>
       </c>
       <c r="E32" s="2" t="n">
         <v>14.75</v>
@@ -2142,10 +2142,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>53.58774456843417</v>
+        <v>53.5877446750235</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>34.09691411825446</v>
+        <v>34.09691412721011</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>1.795983580426009</v>
@@ -2160,7 +2160,7 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>0.09347685506407941</v>
+        <v>0.0934768550125628</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
         <v>44.18436452915455</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>13.92977534151037</v>
+        <v>13.92977540369517</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>1.053801751042616</v>
@@ -2213,7 +2213,7 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>-0.0102843300146885</v>
+        <v>-0.0102843299819899</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
@@ -2251,7 +2251,7 @@
         <v>36.43831637129214</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>21.99582902388497</v>
+        <v>21.99582910455362</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>2.528985684292139</v>
@@ -2301,10 +2301,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>37.29775235181029</v>
+        <v>37.29775226429642</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>27.13297728318202</v>
+        <v>27.13297719712186</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>0.6178356628006788</v>
@@ -2319,7 +2319,7 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>0.3779994403631903</v>
+        <v>0.3779994407752971</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
@@ -2340,7 +2340,7 @@
         <v/>
       </c>
       <c r="D36" s="2" t="n">
-        <v>450.357076267617</v>
+        <v>450.3570762676169</v>
       </c>
       <c r="E36" s="2" t="n">
         <v>74.5</v>
@@ -2354,10 +2354,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>43.20257755502521</v>
+        <v>43.20257747606914</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>8.542082484448462</v>
+        <v>8.542082375698199</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>0.5435439067548555</v>
@@ -2372,7 +2372,7 @@
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>-0.0541424029096032</v>
+        <v>-0.0541424027859738</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
@@ -2407,10 +2407,10 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>49.42826946386565</v>
+        <v>49.42826941589242</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>13.55143727436524</v>
+        <v>13.55143722092805</v>
       </c>
       <c r="J37" s="2" t="n">
         <v>0.5977734942476089</v>
@@ -2425,7 +2425,7 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>-0.085750096914386</v>
+        <v>-0.0857500968731737</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
@@ -2460,10 +2460,10 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>54.70469457080497</v>
+        <v>54.70469487406808</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>22.30187226707582</v>
+        <v>22.3018726441397</v>
       </c>
       <c r="J38" s="2" t="n">
         <v>0.5316251204259922</v>
@@ -2478,7 +2478,7 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>0.0140783796872897</v>
+        <v>0.0140783795203816</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
@@ -2513,10 +2513,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>44.72683621650541</v>
+        <v>44.72683610069753</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>18.44940284513235</v>
+        <v>18.44940280019104</v>
       </c>
       <c r="J39" s="2" t="n">
         <v>0.7415643761119077</v>
@@ -2531,7 +2531,7 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>-0.112225682320523</v>
+        <v>-0.1122256822793139</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
@@ -2566,10 +2566,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>57.08322859267743</v>
+        <v>57.08322822726369</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>17.18057315787357</v>
+        <v>17.18057368936899</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>1.201204532330209</v>
@@ -2584,7 +2584,7 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>0.0574064350294469</v>
+        <v>0.0574064352045982</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
@@ -2619,10 +2619,10 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>50.7310841260519</v>
+        <v>50.7310841029356</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>12.38310166049494</v>
+        <v>12.38310167198658</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>0.7146941047175062</v>
@@ -2658,7 +2658,7 @@
         <v/>
       </c>
       <c r="D42" s="2" t="n">
-        <v>419.1744451668981</v>
+        <v>419.174445166898</v>
       </c>
       <c r="E42" s="2" t="n">
         <v>25.8</v>
@@ -2672,10 +2672,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>55.02449394882009</v>
+        <v>55.02449391742635</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>23.6768871309057</v>
+        <v>23.67688712688496</v>
       </c>
       <c r="J42" s="2" t="n">
         <v>0.9556686811682706</v>
@@ -2725,10 +2725,10 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>23.48532294346204</v>
+        <v>23.48532301472335</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>55.30601209721097</v>
+        <v>55.30601215380953</v>
       </c>
       <c r="J43" s="2" t="n">
         <v>0.7419841596453609</v>
@@ -2743,7 +2743,7 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>0.0029094900209389</v>
+        <v>0.0029094900312419</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
@@ -2764,7 +2764,7 @@
         <v/>
       </c>
       <c r="D44" s="2" t="n">
-        <v>393.175888902694</v>
+        <v>393.1758889026943</v>
       </c>
       <c r="E44" s="2" t="n">
         <v>19.5</v>
@@ -2778,10 +2778,10 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>35.0101092558788</v>
+        <v>35.01010917200365</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>25.931058593161</v>
+        <v>25.93105855792507</v>
       </c>
       <c r="J44" s="2" t="n">
         <v>2.633623604883756</v>
@@ -2796,7 +2796,7 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>-0.0464793444735024</v>
+        <v>-0.0464793444631961</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
@@ -2831,10 +2831,10 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>49.18804479547161</v>
+        <v>49.18804503133477</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>12.27872906767675</v>
+        <v>12.27872909353246</v>
       </c>
       <c r="J45" s="2" t="n">
         <v>0.4851515203636359</v>
@@ -2849,7 +2849,7 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>0.0730598205857405</v>
+        <v>0.0730598204930125</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
@@ -2884,10 +2884,10 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>50.92365407559508</v>
+        <v>50.92365550605701</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>9.806275768982216</v>
+        <v>9.806276713361891</v>
       </c>
       <c r="J46" s="2" t="n">
         <v>0.0747420465119755</v>
@@ -2902,7 +2902,7 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>0.096114608249349</v>
+        <v>0.09611460400455581</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
@@ -2937,10 +2937,10 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>49.76664282805221</v>
+        <v>49.76664279490457</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>15.4819326378806</v>
+        <v>15.48193259133164</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>0.5075576072771187</v>
@@ -2955,7 +2955,7 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>-0.0126520572965968</v>
+        <v>-0.0126520573069006</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
@@ -2976,7 +2976,7 @@
         <v/>
       </c>
       <c r="D48" s="2" t="n">
-        <v>372.9722255578729</v>
+        <v>372.9722255578732</v>
       </c>
       <c r="E48" s="2" t="n">
         <v>13.8</v>
@@ -2990,10 +2990,10 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>52.30168121165394</v>
+        <v>52.30168129203528</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>27.20162786918543</v>
+        <v>27.20162805373186</v>
       </c>
       <c r="J48" s="2" t="n">
         <v>0.3390727924063561</v>
@@ -3008,7 +3008,7 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>0.0022935548433112</v>
+        <v>0.0022935547814944</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
@@ -3061,7 +3061,7 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>0.011318560176068</v>
+        <v>0.0113185601657682</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
@@ -3082,7 +3082,7 @@
         <v/>
       </c>
       <c r="D50" s="2" t="n">
-        <v>364.8107824047813</v>
+        <v>364.8107824047804</v>
       </c>
       <c r="E50" s="2" t="n">
         <v>60</v>
@@ -3096,10 +3096,10 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>52.16489368283852</v>
+        <v>52.1648936802383</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>10.57232561535845</v>
+        <v>10.57232564303941</v>
       </c>
       <c r="J50" s="2" t="n">
         <v>0.3884383752219517</v>
@@ -3114,7 +3114,7 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>1.714778827357518</v>
+        <v>1.714778827295699</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
@@ -3149,10 +3149,10 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>46.58871901396223</v>
+        <v>46.5887190325304</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>24.97273180932224</v>
+        <v>24.97273187999811</v>
       </c>
       <c r="J51" s="2" t="n">
         <v>0.2162454325099041</v>
@@ -3167,7 +3167,7 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>-0.0370862846248416</v>
+        <v>-0.0370862846289644</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
@@ -3202,10 +3202,10 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>50.73631469167056</v>
+        <v>50.73631477243313</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>8.566707783910287</v>
+        <v>8.566707797494177</v>
       </c>
       <c r="J52" s="2" t="n">
         <v>0.6607899626004681</v>
@@ -3220,7 +3220,7 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>-0.0144298795963248</v>
+        <v>-0.0144298796478403</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
@@ -3258,7 +3258,7 @@
         <v>50.93823418234832</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>10.20390864595953</v>
+        <v>10.20390864370355</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>0.1952270638936701</v>
@@ -3273,7 +3273,7 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>0.0675868625162675</v>
+        <v>0.0675868625265706</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
@@ -3294,7 +3294,7 @@
         <v/>
       </c>
       <c r="D54" s="2" t="n">
-        <v>352.1249085842346</v>
+        <v>352.1249085842343</v>
       </c>
       <c r="E54" s="2" t="n">
         <v>0</v>
@@ -3308,10 +3308,10 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>30.33335353128142</v>
+        <v>30.33335353473473</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>24.70963796382662</v>
+        <v>24.70963798295186</v>
       </c>
       <c r="J54" s="2" t="n">
         <v>0</v>
@@ -3326,7 +3326,7 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>-1.047930056869548</v>
+        <v>-1.047930056951973</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
@@ -3361,10 +3361,10 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>42.42273709710385</v>
+        <v>42.42273710004807</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>9.03585733126558</v>
+        <v>9.035857335734343</v>
       </c>
       <c r="J55" s="2" t="n">
         <v>0.3483373997759351</v>
@@ -3379,7 +3379,7 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>-0.0293021760513786</v>
+        <v>-0.0293021761028913</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
@@ -3400,7 +3400,7 @@
         <v/>
       </c>
       <c r="D56" s="2" t="n">
-        <v>344.4726968174038</v>
+        <v>344.4726968174039</v>
       </c>
       <c r="E56" s="2" t="n">
         <v>105.5</v>
@@ -3414,10 +3414,10 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>41.22010919289527</v>
+        <v>41.22010908431373</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>14.01687637347819</v>
+        <v>14.01687644298336</v>
       </c>
       <c r="J56" s="2" t="n">
         <v>1.67872921694417</v>
@@ -3432,7 +3432,7 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>-0.3796153910140771</v>
+        <v>-0.3796153903959114</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
@@ -3467,10 +3467,10 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>48.48313166392384</v>
+        <v>48.48313183366961</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>26.19789054212075</v>
+        <v>26.19789054601214</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>0.3359423949778098</v>
@@ -3520,10 +3520,10 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>28.35692069100982</v>
+        <v>28.35692071737463</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>27.44815137541359</v>
+        <v>27.44815135022232</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>1.653008422598548</v>
@@ -3538,7 +3538,7 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>-0.0139874692416193</v>
+        <v>-0.0139874692519222</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
@@ -3559,7 +3559,7 @@
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>337.5014318014976</v>
+        <v>337.5014318014991</v>
       </c>
       <c r="E59" s="2" t="n">
         <v>26</v>
@@ -3573,10 +3573,10 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>38.6317903313488</v>
+        <v>38.63179023705977</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>27.71108258040195</v>
+        <v>27.71108267960776</v>
       </c>
       <c r="J59" s="2" t="n">
         <v>0.6761643598881846</v>
@@ -3591,7 +3591,7 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>-0.0023915764681421</v>
+        <v>-0.002391576385721</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
@@ -3626,10 +3626,10 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>39.62140688979945</v>
+        <v>39.62140690004976</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>32.55773089204103</v>
+        <v>32.55773091442138</v>
       </c>
       <c r="J60" s="2" t="n">
         <v>0.5852551952054829</v>
@@ -3665,7 +3665,7 @@
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>334.2416530707876</v>
+        <v>334.2416530707877</v>
       </c>
       <c r="E61" s="2" t="n">
         <v>32.65</v>
@@ -3679,10 +3679,10 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>50.76748373407746</v>
+        <v>50.76748480707426</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>8.232681164246451</v>
+        <v>8.232681516660033</v>
       </c>
       <c r="J61" s="2" t="n">
         <v>0.7607929230308067</v>
@@ -3697,7 +3697,7 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>0.0384647188495408</v>
+        <v>0.0384647182931859</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
@@ -3718,7 +3718,7 @@
         <v/>
       </c>
       <c r="D62" s="2" t="n">
-        <v>333.0183763969388</v>
+        <v>333.0183763969389</v>
       </c>
       <c r="E62" s="2" t="n">
         <v>14.75</v>
@@ -3732,10 +3732,10 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>24.76761666148377</v>
+        <v>24.76761654329372</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>24.9465641163318</v>
+        <v>24.9465641585789</v>
       </c>
       <c r="J62" s="2" t="n">
         <v>3.092441738586137</v>
@@ -3750,7 +3750,7 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>-0.1118197576540327</v>
+        <v>-0.1118197576025184</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
@@ -3771,7 +3771,7 @@
         <v/>
       </c>
       <c r="D63" s="2" t="n">
-        <v>331.4637963577784</v>
+        <v>331.4637963577783</v>
       </c>
       <c r="E63" s="2" t="n">
         <v>27.7</v>
@@ -3785,10 +3785,10 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>32.41645748888907</v>
+        <v>32.41645746766615</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>19.27713960663537</v>
+        <v>19.27713964822369</v>
       </c>
       <c r="J63" s="2" t="n">
         <v>0.951770542148195</v>
@@ -3803,7 +3803,7 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>-0.2440892927937312</v>
+        <v>-0.2440892928555463</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
@@ -3838,10 +3838,10 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>39.89126307860599</v>
+        <v>39.89126324080706</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>16.13051192245653</v>
+        <v>16.13051195168057</v>
       </c>
       <c r="J64" s="2" t="n">
         <v>0.7020971486000142</v>
@@ -3856,7 +3856,7 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>-0.1374133380784252</v>
+        <v>-0.1374133380681245</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
@@ -3877,7 +3877,7 @@
         <v/>
       </c>
       <c r="D65" s="2" t="n">
-        <v>322.1183274563289</v>
+        <v>322.1183274563284</v>
       </c>
       <c r="E65" s="2" t="n">
         <v>68.5</v>
@@ -3891,10 +3891,10 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>43.23004439744802</v>
+        <v>43.23004444130681</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>15.93433186530655</v>
+        <v>15.93433192821562</v>
       </c>
       <c r="J65" s="2" t="n">
         <v>0.7089900705847003</v>
@@ -3909,7 +3909,7 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>-0.3721517096958779</v>
+        <v>-0.3721517101080017</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
@@ -3944,10 +3944,10 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>44.62162333988528</v>
+        <v>44.62162323283446</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>21.31044172031665</v>
+        <v>21.31044175539902</v>
       </c>
       <c r="J66" s="2" t="n">
         <v>0.5345146938859737</v>
@@ -3962,7 +3962,7 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>-0.0544585819252956</v>
+        <v>-0.0544585818943868</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
@@ -3997,10 +3997,10 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>44.31603431326939</v>
+        <v>44.31604735532043</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>22.81993488272189</v>
+        <v>22.81993943831284</v>
       </c>
       <c r="J67" s="2" t="n">
         <v>0.4719151337708807</v>
@@ -4015,7 +4015,7 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>0.0012891737087281</v>
+        <v>0.0012891706281601</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
@@ -4050,7 +4050,7 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>43.16358179864906</v>
+        <v>43.16358200312141</v>
       </c>
       <c r="I68" s="2" t="n">
         <v>10.65137082042527</v>
@@ -4068,7 +4068,7 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>-0.0169469591795851</v>
+        <v>-0.0169469592001902</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
@@ -4089,7 +4089,7 @@
         <v/>
       </c>
       <c r="D69" s="2" t="n">
-        <v>310.427635276651</v>
+        <v>310.4276352766508</v>
       </c>
       <c r="E69" s="2" t="n">
         <v>17.1</v>
@@ -4103,10 +4103,10 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>43.29169737585897</v>
+        <v>43.29169746622856</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>18.63885063998946</v>
+        <v>18.6388506235312</v>
       </c>
       <c r="J69" s="2" t="n">
         <v>0.911360284080754</v>
@@ -4121,7 +4121,7 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>0.0005311494069418</v>
+        <v>0.0005311493863374</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
@@ -4156,10 +4156,10 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>43.14906620416949</v>
+        <v>43.14906615127083</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>23.50223984498413</v>
+        <v>23.50223988705314</v>
       </c>
       <c r="J70" s="2" t="n">
         <v>0.5120523351121652</v>
@@ -4174,7 +4174,7 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>0.1264880515905116</v>
+        <v>0.1264880517141436</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
@@ -4209,7 +4209,7 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>44.43546668014309</v>
+        <v>44.43546668675432</v>
       </c>
       <c r="I71" s="2" t="n">
         <v>18.87600789052682</v>
@@ -4227,7 +4227,7 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>-0.1577845763663179</v>
+        <v>-0.1577845764281358</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
@@ -4248,7 +4248,7 @@
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>297.8901220404101</v>
+        <v>297.8901220404103</v>
       </c>
       <c r="E72" s="2" t="n">
         <v>13.05</v>
@@ -4262,10 +4262,10 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>44.63866019244454</v>
+        <v>44.63866022279278</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>20.77728971900297</v>
+        <v>20.77728980728407</v>
       </c>
       <c r="J72" s="2" t="n">
         <v>0.502963476140964</v>
@@ -4280,7 +4280,7 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>3.172226460564781e-05</v>
+        <v>3.172225430302794e-05</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
@@ -4315,10 +4315,10 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>51.56782478579483</v>
+        <v>51.5678248157296</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>12.99633619565235</v>
+        <v>12.99633628037481</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>1.603768348902477</v>
@@ -4333,7 +4333,7 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>-0.0309995603711438</v>
+        <v>-0.0309995603814466</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
@@ -4354,7 +4354,7 @@
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>292.9792414255554</v>
+        <v>292.9792414255561</v>
       </c>
       <c r="E74" s="2" t="n">
         <v>699</v>
@@ -4368,10 +4368,10 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>44.12876807303724</v>
+        <v>44.12876814630479</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>11.31046960697478</v>
+        <v>11.31046961010666</v>
       </c>
       <c r="J74" s="2" t="n">
         <v>0.4262569204174543</v>
@@ -4386,7 +4386,7 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>-2.325496129776147</v>
+        <v>-2.325496132454834</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
@@ -4407,7 +4407,7 @@
         <v/>
       </c>
       <c r="D75" s="2" t="n">
-        <v>292.2727637231952</v>
+        <v>292.2727637231951</v>
       </c>
       <c r="E75" s="2" t="n">
         <v>276.5</v>
@@ -4421,10 +4421,10 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>27.60065125312337</v>
+        <v>27.6006514368144</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>39.5913450503996</v>
+        <v>39.59134505989268</v>
       </c>
       <c r="J75" s="2" t="n">
         <v>1.101667727907232</v>
@@ -4439,7 +4439,7 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>-0.7220464001343458</v>
+        <v>-0.7220464013706298</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>290.5563946990527</v>
+        <v>290.5563946990526</v>
       </c>
       <c r="E76" s="2" t="n">
         <v>9.970000000000001</v>
@@ -4474,10 +4474,10 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>39.69797755024023</v>
+        <v>39.69797596997519</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>22.84733803930289</v>
+        <v>22.84733814630626</v>
       </c>
       <c r="J76" s="2" t="n">
         <v>0.4376298873520786</v>
@@ -4492,7 +4492,7 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>0.0090585002101527</v>
+        <v>0.009058500241062599</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
@@ -4513,7 +4513,7 @@
         <v/>
       </c>
       <c r="D77" s="2" t="n">
-        <v>284.5936052404758</v>
+        <v>284.5936052404757</v>
       </c>
       <c r="E77" s="2" t="n">
         <v>26.65</v>
@@ -4527,10 +4527,10 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>48.14675888224799</v>
+        <v>48.14675887273457</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>22.71983742039029</v>
+        <v>22.71983757968933</v>
       </c>
       <c r="J77" s="2" t="n">
         <v>0.5794892233667036</v>
@@ -4545,7 +4545,7 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>0.1215759977745007</v>
+        <v>0.1215759979187395</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
@@ -4580,10 +4580,10 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>51.21739120138025</v>
+        <v>51.21739120090434</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>11.48208650327126</v>
+        <v>11.48208651725725</v>
       </c>
       <c r="J78" s="2" t="n">
         <v>1.508667725671662</v>
@@ -4598,7 +4598,7 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>0.6964450159931144</v>
+        <v>0.6964450160034265</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
@@ -4633,10 +4633,10 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>36.72531338978541</v>
+        <v>36.72531320496911</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>37.98356625873164</v>
+        <v>37.98356660496544</v>
       </c>
       <c r="J79" s="2" t="n">
         <v>0.7091782403611994</v>
@@ -4651,7 +4651,7 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>0.3264349114034752</v>
+        <v>0.3264349120216505</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
@@ -4672,7 +4672,7 @@
         <v/>
       </c>
       <c r="D80" s="2" t="n">
-        <v>264.66307813358</v>
+        <v>264.6630781335797</v>
       </c>
       <c r="E80" s="2" t="n">
         <v>47</v>
@@ -4686,10 +4686,10 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>42.71665610596107</v>
+        <v>42.71665586666957</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>9.140662847124412</v>
+        <v>9.140662893558956</v>
       </c>
       <c r="J80" s="2" t="n">
         <v>0.918806715129435</v>
@@ -4704,7 +4704,7 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>-0.0378001686748628</v>
+        <v>-0.0378001681185071</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
@@ -4739,10 +4739,10 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>50.21515309932448</v>
+        <v>50.21515326515548</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>12.34245574662815</v>
+        <v>12.34245617887821</v>
       </c>
       <c r="J81" s="2" t="n">
         <v>0.4095651925805789</v>
@@ -4757,7 +4757,7 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>-0.012616557779775</v>
+        <v>-0.0126165578931077</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
@@ -4792,10 +4792,10 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>45.35370197292813</v>
+        <v>45.35370215381646</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>16.77278618428673</v>
+        <v>16.77278616033155</v>
       </c>
       <c r="J82" s="2" t="n">
         <v>0.4670247023880471</v>
@@ -4810,7 +4810,7 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>-0.2187264450002918</v>
+        <v>-0.2187264451033156</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
@@ -4845,10 +4845,10 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>31.90709045651516</v>
+        <v>31.90709043628356</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>22.61088599681586</v>
+        <v>22.6108859698442</v>
       </c>
       <c r="J83" s="2" t="n">
         <v>1.267694664083302</v>
@@ -4898,10 +4898,10 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>40.38847242648038</v>
+        <v>40.38847264881744</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>32.06027482614487</v>
+        <v>32.06027476096221</v>
       </c>
       <c r="J84" s="2" t="n">
         <v>0.6225557950428553</v>
@@ -4937,7 +4937,7 @@
         <v/>
       </c>
       <c r="D85" s="2" t="n">
-        <v>251.6014864706753</v>
+        <v>251.6014864706743</v>
       </c>
       <c r="E85" s="2" t="n">
         <v>66</v>
@@ -4951,10 +4951,10 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>48.3759111283575</v>
+        <v>48.37591118037257</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>12.05625700059126</v>
+        <v>12.05625701010428</v>
       </c>
       <c r="J85" s="2" t="n">
         <v>0.2763589828495598</v>
@@ -4969,7 +4969,7 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>-0.1251747436752714</v>
+        <v>-0.125174743737088</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
@@ -5004,10 +5004,10 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>39.65414004088515</v>
+        <v>39.6541399191126</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>7.5580309168634</v>
+        <v>7.558030916863396</v>
       </c>
       <c r="J86" s="2" t="n">
         <v>2.986749443468509</v>
@@ -5022,7 +5022,7 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>0.0146174883231166</v>
+        <v>0.0146174883849338</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
@@ -5043,7 +5043,7 @@
         <v/>
       </c>
       <c r="D87" s="2" t="n">
-        <v>247.4306371673675</v>
+        <v>247.4306371673674</v>
       </c>
       <c r="E87" s="2" t="n">
         <v>10.8</v>
@@ -5060,7 +5060,7 @@
         <v>33.06635877516952</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>23.3368946476919</v>
+        <v>23.33689467604703</v>
       </c>
       <c r="J87" s="2" t="n">
         <v>0.4179182929817769</v>
@@ -5110,10 +5110,10 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>48.71433749644433</v>
+        <v>48.71433743579543</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>5.930345808802407</v>
+        <v>5.930345847115438</v>
       </c>
       <c r="J88" s="2" t="n">
         <v>0.436274081950618</v>
@@ -5128,7 +5128,7 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>0.0415502903731948</v>
+        <v>0.0415502904453151</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
@@ -5163,10 +5163,10 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>43.8817042657624</v>
+        <v>43.88170428445039</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>15.0818304795585</v>
+        <v>15.08183058431626</v>
       </c>
       <c r="J89" s="2" t="n">
         <v>0.5186073575128568</v>
@@ -5181,7 +5181,7 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>0.0155526809337908</v>
+        <v>0.0155526809358521</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
@@ -5219,7 +5219,7 @@
         <v>42.16577189361502</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>10.2949763215147</v>
+        <v>10.29497635124557</v>
       </c>
       <c r="J90" s="2" t="n">
         <v>0.168613957688645</v>
@@ -5234,7 +5234,7 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>0.031078309207495</v>
+        <v>0.0310783092013129</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
@@ -5255,7 +5255,7 @@
         <v/>
       </c>
       <c r="D91" s="2" t="n">
-        <v>232.4316965804152</v>
+        <v>232.4316965804149</v>
       </c>
       <c r="E91" s="2" t="n">
         <v>102</v>
@@ -5269,10 +5269,10 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>49.16387781592628</v>
+        <v>49.16387774062459</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>14.44930207695184</v>
+        <v>14.44930207460586</v>
       </c>
       <c r="J91" s="2" t="n">
         <v>1.351277911539894</v>
@@ -5287,7 +5287,7 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>0.3594726392573232</v>
+        <v>0.3594726396694385</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
@@ -5322,10 +5322,10 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>34.03165126832047</v>
+        <v>34.03165134729996</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>24.15595550586509</v>
+        <v>24.15595550882902</v>
       </c>
       <c r="J92" s="2" t="n">
         <v>0.2697946046931946</v>
@@ -5340,7 +5340,7 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>-0.0216342540739243</v>
+        <v>-0.0216342541357427</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
@@ -5375,10 +5375,10 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>32.59704691572874</v>
+        <v>32.59704687693366</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>29.78140831715586</v>
+        <v>29.78140838246116</v>
       </c>
       <c r="J93" s="2" t="n">
         <v>0.9539468689393882</v>
@@ -5393,7 +5393,7 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>-0.0478241144263929</v>
+        <v>-0.0478241144160887</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
@@ -5431,7 +5431,7 @@
         <v>46.59781347622856</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>14.55126456953445</v>
+        <v>14.5512646240608</v>
       </c>
       <c r="J94" s="2" t="n">
         <v>0.5180395055277867</v>
@@ -5446,7 +5446,7 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>-0.24152616081207</v>
+        <v>-0.241526160709038</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
@@ -5481,10 +5481,10 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>43.75689453703884</v>
+        <v>43.75689456264242</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>14.52606952527272</v>
+        <v>14.52606955811724</v>
       </c>
       <c r="J95" s="2" t="n">
         <v>1.061136792964763</v>
@@ -5499,7 +5499,7 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>-0.008398986498580299</v>
+        <v>-0.0083989865191862</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
@@ -5534,10 +5534,10 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>48.64578567582122</v>
+        <v>48.6457856648475</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>12.18296457283881</v>
+        <v>12.18296464062828</v>
       </c>
       <c r="J96" s="2" t="n">
         <v>0.2249250096795675</v>
@@ -5552,7 +5552,7 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>-0.0838127958451875</v>
+        <v>-0.08381279588639851</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
@@ -5587,10 +5587,10 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>33.17979778344731</v>
+        <v>33.17979786824418</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>8.769809614254433</v>
+        <v>8.769809602556821</v>
       </c>
       <c r="J97" s="2" t="n">
         <v>0.7535309221377681</v>
@@ -5605,7 +5605,7 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>-0.4561794849406828</v>
+        <v>-0.4561794846315825</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
@@ -5640,7 +5640,7 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>40.61848543601389</v>
+        <v>40.61848534278261</v>
       </c>
       <c r="I98" s="2" t="n">
         <v>17.86580193502385</v>
@@ -5693,10 +5693,10 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>50.91200453318152</v>
+        <v>50.91200446564194</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>8.920657514251682</v>
+        <v>8.92065751425168</v>
       </c>
       <c r="J99" s="2" t="n">
         <v>0.603459583538285</v>
@@ -5711,7 +5711,7 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>0.3059918048370221</v>
+        <v>0.3059918046846929</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
@@ -5746,10 +5746,10 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>34.86046143660859</v>
+        <v>34.86046120086584</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>32.47825081832897</v>
+        <v>32.47825076977574</v>
       </c>
       <c r="J100" s="2" t="n">
         <v>0.7728841266485443</v>
@@ -5764,7 +5764,7 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>0.0029119068377951</v>
+        <v>0.002911906848098</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
@@ -5802,7 +5802,7 @@
         <v>41.08444409117836</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>10.97575315166562</v>
+        <v>10.97575308408577</v>
       </c>
       <c r="J101" s="2" t="n">
         <v>0.8187801994017417</v>
@@ -5817,7 +5817,7 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>0.0050552602008418</v>
+        <v>0.0050552602111418</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
@@ -5852,10 +5852,10 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>39.5403749382553</v>
+        <v>39.5403746782918</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>23.16157988497739</v>
+        <v>23.16158012845588</v>
       </c>
       <c r="J102" s="2" t="n">
         <v>0.6938625427939001</v>
@@ -5870,7 +5870,7 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>-0.0581086236187191</v>
+        <v>-0.0581086230829653</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
@@ -5891,7 +5891,7 @@
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>210.8729195606529</v>
+        <v>210.8729195606531</v>
       </c>
       <c r="E103" s="2" t="n">
         <v>23.05</v>
@@ -5905,10 +5905,10 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>45.25963939602129</v>
+        <v>45.25963943182494</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>5.119036127622759</v>
+        <v>5.119036154578149</v>
       </c>
       <c r="J103" s="2" t="n">
         <v>0.8622069614414106</v>
@@ -5923,7 +5923,7 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>-0.0033726784275606</v>
+        <v>-0.0033726784687696</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
@@ -5961,7 +5961,7 @@
         <v>50.43547673679654</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>18.06665914057961</v>
+        <v>18.06665908503258</v>
       </c>
       <c r="J104" s="2" t="n">
         <v>0.9288049767465556</v>
@@ -5997,7 +5997,7 @@
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>194.2179619016075</v>
+        <v>194.2179619016106</v>
       </c>
       <c r="E105" s="2" t="n">
         <v>64.40000000000001</v>
@@ -6011,10 +6011,10 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>51.18018452391785</v>
+        <v>51.18018451381249</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>21.54249097412362</v>
+        <v>21.542490833729</v>
       </c>
       <c r="J105" s="2" t="n">
         <v>1.504848647200643</v>
@@ -6029,7 +6029,7 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>-1.184543157910109</v>
+        <v>-1.184543157539203</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
@@ -6064,10 +6064,10 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>42.75937490525939</v>
+        <v>42.75937508015001</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>16.36644319748243</v>
+        <v>16.36644321871258</v>
       </c>
       <c r="J106" s="2" t="n">
         <v>1.081609927212568</v>
@@ -6082,7 +6082,7 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>0.0069930216143574</v>
+        <v>0.0069930215937528</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
@@ -6117,10 +6117,10 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>45.46547026813975</v>
+        <v>45.46547030186201</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>13.19563537735114</v>
+        <v>13.19563541064757</v>
       </c>
       <c r="J107" s="2" t="n">
         <v>0.5325164438786336</v>
@@ -6135,7 +6135,7 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>-0.0114865284899529</v>
+        <v>-0.0114865286135915</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
@@ -6156,7 +6156,7 @@
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>177.8432355317165</v>
+        <v>177.8432355317164</v>
       </c>
       <c r="E108" s="2" t="n">
         <v>196</v>
@@ -6170,7 +6170,7 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>43.30531210020706</v>
+        <v>43.30531215740378</v>
       </c>
       <c r="I108" s="2" t="n">
         <v>10.00399064412504</v>
@@ -6223,10 +6223,10 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>48.39438040279474</v>
+        <v>48.39437996819087</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>12.5414528936279</v>
+        <v>12.54145300237842</v>
       </c>
       <c r="J109" s="2" t="n">
         <v>0.5535224586928081</v>
@@ -6241,7 +6241,7 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>0.0512900794089901</v>
+        <v>0.0512900796150477</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
@@ -6276,7 +6276,7 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>52.77989777201535</v>
+        <v>52.77989777541445</v>
       </c>
       <c r="I110" s="2" t="n">
         <v>9.1671226089423</v>
@@ -6294,7 +6294,7 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>2.690341496505717</v>
+        <v>2.690341496361478</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
@@ -6332,7 +6332,7 @@
         <v>45.75353411473413</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>11.43605780234731</v>
+        <v>11.43605779883075</v>
       </c>
       <c r="J111" s="2" t="n">
         <v>0.0001400550416313</v>
@@ -6385,7 +6385,7 @@
         <v>51.91879873819772</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>19.44384807920188</v>
+        <v>19.44384807457648</v>
       </c>
       <c r="J112" s="2" t="n">
         <v>0.2236906510034263</v>
@@ -6400,7 +6400,7 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>0.0404375592194801</v>
+        <v>0.040437559178269</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
@@ -6435,10 +6435,10 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>47.78896417967887</v>
+        <v>47.78896365929295</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>15.68770208826056</v>
+        <v>15.68770203533845</v>
       </c>
       <c r="J113" s="2" t="n">
         <v>1.138063168865906</v>
@@ -6453,7 +6453,7 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>0.0102298855288995</v>
+        <v>0.0102298858998013</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
@@ -6474,7 +6474,7 @@
         <v/>
       </c>
       <c r="D114" s="2" t="n">
-        <v>161.8770216573484</v>
+        <v>161.8770216573474</v>
       </c>
       <c r="E114" s="2" t="n">
         <v>26.7</v>
@@ -6488,10 +6488,10 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>32.86232829554959</v>
+        <v>32.86232830231734</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>19.10831854223087</v>
+        <v>19.10831852076622</v>
       </c>
       <c r="J114" s="2" t="n">
         <v>0.3016058633221153</v>
@@ -6506,7 +6506,7 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>-0.1218205302396243</v>
+        <v>-0.1218205302602301</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
@@ -6541,10 +6541,10 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>49.90280746149206</v>
+        <v>49.90280756175169</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>12.69467963153254</v>
+        <v>12.69467972535677</v>
       </c>
       <c r="J115" s="2" t="n">
         <v>1.087615949355959</v>
@@ -6559,7 +6559,7 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-0.0005648757909755</v>
+        <v>-0.0005648758012771</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
@@ -6594,10 +6594,10 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>38.80466856445916</v>
+        <v>38.80466804510702</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>9.519760066748011</v>
+        <v>9.51976021130945</v>
       </c>
       <c r="J116" s="2" t="n">
         <v>0.9554569055577288</v>
@@ -6612,7 +6612,7 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>0.0102867784494589</v>
+        <v>0.0102867785153978</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
@@ -6647,10 +6647,10 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>41.02453311432241</v>
+        <v>41.02453300258299</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>10.16589349199025</v>
+        <v>10.16589351099681</v>
       </c>
       <c r="J117" s="2" t="n">
         <v>0.1011474815970939</v>
@@ -6665,7 +6665,7 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>-0.0017563047307236</v>
+        <v>-0.0017563047101163</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
@@ -6700,10 +6700,10 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>36.77541197846822</v>
+        <v>36.77541204876096</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>23.0372737273773</v>
+        <v>23.03727374614221</v>
       </c>
       <c r="J118" s="2" t="n">
         <v>0.1997971702293157</v>
@@ -6718,7 +6718,7 @@
         <v>-1</v>
       </c>
       <c r="N118" s="2" t="n">
-        <v>-0.0115572104005615</v>
+        <v>-0.0115572104211656</v>
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
@@ -6753,10 +6753,10 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>37.80698432934248</v>
+        <v>37.80698450167327</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>17.25404834173696</v>
+        <v>17.25404851467422</v>
       </c>
       <c r="J119" s="2" t="n">
         <v>0.09485171628344451</v>
@@ -6771,7 +6771,7 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>-0.014061397039644</v>
+        <v>-0.0140613970190381</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
@@ -6806,10 +6806,10 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>39.10305944947053</v>
+        <v>39.10305957349571</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>15.84860772938364</v>
+        <v>15.84860774067127</v>
       </c>
       <c r="J120" s="2" t="n">
         <v>0.2898815301299903</v>
@@ -6824,7 +6824,7 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>0.0639195305219997</v>
+        <v>0.06391953048078711</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
@@ -6845,7 +6845,7 @@
         <v/>
       </c>
       <c r="D121" s="2" t="n">
-        <v>150.6907412260265</v>
+        <v>150.6907412260264</v>
       </c>
       <c r="E121" s="2" t="n">
         <v>79.59999999999999</v>
@@ -6859,10 +6859,10 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>41.33665312453917</v>
+        <v>41.33665306039034</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>10.76942217858215</v>
+        <v>10.76942234848532</v>
       </c>
       <c r="J121" s="2" t="n">
         <v>0.5036580712732786</v>
@@ -6877,7 +6877,7 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>0.1293157686558813</v>
+        <v>0.1293157691710231</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
@@ -6912,10 +6912,10 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>46.1734966564245</v>
+        <v>46.17349648567914</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>8.802496416839771</v>
+        <v>8.802496472927102</v>
       </c>
       <c r="J122" s="2" t="n">
         <v>0.3445227478682101</v>
@@ -6930,7 +6930,7 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>0.0059497130093179</v>
+        <v>0.005949713040227</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
@@ -6951,7 +6951,7 @@
         <v/>
       </c>
       <c r="D123" s="2" t="n">
-        <v>143.216443171296</v>
+        <v>143.2164431712961</v>
       </c>
       <c r="E123" s="2" t="n">
         <v>14.35</v>
@@ -6965,10 +6965,10 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>47.14649695124344</v>
+        <v>47.14649688258773</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>11.92050054080074</v>
+        <v>11.92050045338421</v>
       </c>
       <c r="J123" s="2" t="n">
         <v>0.5152589055244483</v>
@@ -6983,7 +6983,7 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>-0.0076900530347278</v>
+        <v>-0.0076900530141223</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
@@ -7018,10 +7018,10 @@
         <v>0</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>43.64610467316226</v>
+        <v>43.64610464171341</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>19.23217670651324</v>
+        <v>19.23217675365634</v>
       </c>
       <c r="J124" s="2" t="n">
         <v>0.1051216414652538</v>
@@ -7036,7 +7036,7 @@
         <v>-1</v>
       </c>
       <c r="N124" s="2" t="n">
-        <v>0.0159319404163587</v>
+        <v>0.0159319405502945</v>
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
@@ -7071,10 +7071,10 @@
         <v>0</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>36.18091045899258</v>
+        <v>36.18091053745876</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>9.354981190098441</v>
+        <v>9.354981228073022</v>
       </c>
       <c r="J125" s="2" t="n">
         <v>0.2862937149337433</v>
@@ -7089,7 +7089,7 @@
         <v>-1</v>
       </c>
       <c r="N125" s="2" t="n">
-        <v>-0.0036221740890226</v>
+        <v>-0.0036221741302361</v>
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>
@@ -7124,10 +7124,10 @@
         <v>0</v>
       </c>
       <c r="H126" s="2" t="n">
-        <v>39.06292275115396</v>
+        <v>39.06292270622599</v>
       </c>
       <c r="I126" s="2" t="n">
-        <v>9.452739815720539</v>
+        <v>9.452739850796</v>
       </c>
       <c r="J126" s="2" t="n">
         <v>0.7371579717980277</v>
@@ -7142,7 +7142,7 @@
         <v>-1</v>
       </c>
       <c r="N126" s="2" t="n">
-        <v>-0.0005736163216236</v>
+        <v>-0.0005736163092595001</v>
       </c>
       <c r="O126" s="2" t="inlineStr">
         <is>
@@ -7177,10 +7177,10 @@
         <v>0</v>
       </c>
       <c r="H127" s="2" t="n">
-        <v>50.9273266867197</v>
+        <v>50.927326741284</v>
       </c>
       <c r="I127" s="2" t="n">
-        <v>10.55419107212293</v>
+        <v>10.55419107618756</v>
       </c>
       <c r="J127" s="2" t="n">
         <v>0.7333678287830576</v>
@@ -7195,7 +7195,7 @@
         <v>-1</v>
       </c>
       <c r="N127" s="2" t="n">
-        <v>-0.0101972522726693</v>
+        <v>-0.0101972522932754</v>
       </c>
       <c r="O127" s="2" t="inlineStr">
         <is>
@@ -7230,10 +7230,10 @@
         <v>0</v>
       </c>
       <c r="H128" s="2" t="n">
-        <v>39.96116768194389</v>
+        <v>39.96116754927892</v>
       </c>
       <c r="I128" s="2" t="n">
-        <v>18.30873215953499</v>
+        <v>18.30873243307893</v>
       </c>
       <c r="J128" s="2" t="n">
         <v>0.5127334465195246</v>
@@ -7248,7 +7248,7 @@
         <v>-1</v>
       </c>
       <c r="N128" s="2" t="n">
-        <v>0.0015208744634838</v>
+        <v>0.0015208746901456</v>
       </c>
       <c r="O128" s="2" t="inlineStr">
         <is>
@@ -7283,10 +7283,10 @@
         <v>0</v>
       </c>
       <c r="H129" s="2" t="n">
-        <v>41.89733815074717</v>
+        <v>41.89733806673743</v>
       </c>
       <c r="I129" s="2" t="n">
-        <v>14.10139027183106</v>
+        <v>14.10139034621174</v>
       </c>
       <c r="J129" s="2" t="n">
         <v>0.9779548285610944</v>
@@ -7301,7 +7301,7 @@
         <v>-1</v>
       </c>
       <c r="N129" s="2" t="n">
-        <v>-0.0484924271076976</v>
+        <v>-0.0484924270252753</v>
       </c>
       <c r="O129" s="2" t="inlineStr">
         <is>
@@ -7322,7 +7322,7 @@
         <v/>
       </c>
       <c r="D130" s="2" t="n">
-        <v>89.49831170708894</v>
+        <v>89.49831170708893</v>
       </c>
       <c r="E130" s="2" t="n">
         <v>45.6</v>
@@ -7339,7 +7339,7 @@
         <v>49.14989578507964</v>
       </c>
       <c r="I130" s="2" t="n">
-        <v>13.93374916693373</v>
+        <v>13.93374915212161</v>
       </c>
       <c r="J130" s="2" t="n">
         <v>0.7975212146144058</v>
@@ -7375,7 +7375,7 @@
         <v/>
       </c>
       <c r="D131" s="2" t="n">
-        <v>88.34879135601571</v>
+        <v>88.3487913560156</v>
       </c>
       <c r="E131" s="2" t="n">
         <v>9.4</v>
@@ -7389,10 +7389,10 @@
         <v>0</v>
       </c>
       <c r="H131" s="2" t="n">
-        <v>42.81461567884486</v>
+        <v>42.81461527802914</v>
       </c>
       <c r="I131" s="2" t="n">
-        <v>15.5558706878708</v>
+        <v>15.55587129457165</v>
       </c>
       <c r="J131" s="2" t="n">
         <v>0.5619201813244366</v>
@@ -7407,7 +7407,7 @@
         <v>-1</v>
       </c>
       <c r="N131" s="2" t="n">
-        <v>-0.008275869476349</v>
+        <v>-0.008275869332108899</v>
       </c>
       <c r="O131" s="2" t="inlineStr">
         <is>
@@ -7442,10 +7442,10 @@
         <v>0</v>
       </c>
       <c r="H132" s="2" t="n">
-        <v>51.74505613837026</v>
+        <v>51.74505581842296</v>
       </c>
       <c r="I132" s="2" t="n">
-        <v>11.77863272633815</v>
+        <v>11.7786327326755</v>
       </c>
       <c r="J132" s="2" t="n">
         <v>0.6524428229882353</v>
@@ -7460,7 +7460,7 @@
         <v>-1</v>
       </c>
       <c r="N132" s="2" t="n">
-        <v>0.016034486672102</v>
+        <v>0.0160344867030118</v>
       </c>
       <c r="O132" s="2" t="inlineStr">
         <is>
@@ -7495,10 +7495,10 @@
         <v>0</v>
       </c>
       <c r="H133" s="2" t="n">
-        <v>44.53314503206301</v>
+        <v>44.53314504609418</v>
       </c>
       <c r="I133" s="2" t="n">
-        <v>12.80569380572918</v>
+        <v>12.80569386850856</v>
       </c>
       <c r="J133" s="2" t="n">
         <v>0.2469258623831483</v>
@@ -7513,7 +7513,7 @@
         <v>-1</v>
       </c>
       <c r="N133" s="2" t="n">
-        <v>-0.0580568853523309</v>
+        <v>-0.0580568853626315</v>
       </c>
       <c r="O133" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
scan: seg0 2026-09-29 00:38 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq1_2026-09-24.xlsx
+++ b/output/full_scan/batch_seq1_2026-09-24.xlsx
@@ -552,7 +552,7 @@
         <v>0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>76.76980525541725</v>
+        <v>76.76980524038702</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>31.4168015702786</v>
@@ -570,7 +570,7 @@
         <v>-1</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>24.49570838768908</v>
+        <v>24.49570838713284</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -605,10 +605,10 @@
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>79.89106143081827</v>
+        <v>79.89106144724846</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>53.06968890241327</v>
+        <v>53.06968897342369</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>2.741649652972179</v>
@@ -623,7 +623,7 @@
         <v>-1</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>1.590931853720629</v>
+        <v>1.590931853431317</v>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
@@ -658,10 +658,10 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>58.61440598226877</v>
+        <v>58.61440390091276</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>17.18896536541293</v>
+        <v>17.18896616509328</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>1.283795586748832</v>
@@ -676,7 +676,7 @@
         <v>-1</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>0.0340843738862658</v>
+        <v>0.034084376612413</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
@@ -711,7 +711,7 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>56.55433808511896</v>
+        <v>56.55433813085726</v>
       </c>
       <c r="I5" s="2" t="n">
         <v>40.34462239767203</v>
@@ -729,7 +729,7 @@
         <v>-1</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>-0.0751935973454885</v>
+        <v>-0.0751935973521636</v>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
@@ -750,7 +750,7 @@
         <v/>
       </c>
       <c r="D6" s="2" t="n">
-        <v>767.8038587209888</v>
+        <v>767.8038587209887</v>
       </c>
       <c r="E6" s="2" t="n">
         <v>35.7</v>
@@ -764,10 +764,10 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>60.93299614592757</v>
+        <v>60.93299628370752</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>26.89643566749574</v>
+        <v>26.89643574083017</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>0.999049460502734</v>
@@ -782,7 +782,7 @@
         <v>-1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>0.0082772938571382</v>
+        <v>0.0082772937792526</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
@@ -803,7 +803,7 @@
         <v/>
       </c>
       <c r="D7" s="2" t="n">
-        <v>739.1887917528753</v>
+        <v>739.1887917528754</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>238</v>
@@ -817,10 +817,10 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>58.09717154455284</v>
+        <v>58.09717155545822</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>23.99712473988518</v>
+        <v>23.99712475800661</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>0.7949632640336151</v>
@@ -835,7 +835,7 @@
         <v>-1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>-1.694069483463693</v>
+        <v>-1.694069483652855</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
@@ -870,10 +870,10 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>75.49115445273235</v>
+        <v>75.49115435857719</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>45.93921664763305</v>
+        <v>45.93921666616041</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>0.3006969482605902</v>
@@ -888,7 +888,7 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>0.06822995720925989</v>
+        <v>0.06822995725377499</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
@@ -923,10 +923,10 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>65.72105379229193</v>
+        <v>65.72105380200219</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>37.09592363131511</v>
+        <v>37.09592355373212</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>0.7737003345632983</v>
@@ -941,7 +941,7 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>0.4556074240692371</v>
+        <v>0.4556074240469865</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
@@ -994,7 +994,7 @@
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>-0.0569605197490807</v>
+        <v>-0.0569605197300099</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
@@ -1029,10 +1029,10 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>58.52601513452927</v>
+        <v>58.52601507359403</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>31.75787830596096</v>
+        <v>31.75787825517412</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>0.6525081178999347</v>
@@ -1047,7 +1047,7 @@
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>0.09325906346322931</v>
+        <v>0.0932590635299913</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
@@ -1082,10 +1082,10 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>60.71553072717938</v>
+        <v>60.71553058892556</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>34.27801534311887</v>
+        <v>34.2780154588573</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>0.4865206968699114</v>
@@ -1100,7 +1100,7 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>-0.341278136417837</v>
+        <v>-0.3412781364559758</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>60.28988319413902</v>
+        <v>60.28988236524086</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>18.11439463217432</v>
+        <v>18.11439440416688</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>1.438336874983999</v>
@@ -1153,7 +1153,7 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>0.0821446363620538</v>
+        <v>0.0821446368405189</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
@@ -1188,7 +1188,7 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>53.53620403183438</v>
+        <v>53.53620410186679</v>
       </c>
       <c r="I14" s="2" t="n">
         <v>21.43000327057417</v>
@@ -1206,7 +1206,7 @@
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>0.001400773993717</v>
+        <v>0.0014007739825906</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
@@ -1241,10 +1241,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>52.08992669373536</v>
+        <v>52.08992664370918</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>10.26933187518033</v>
+        <v>10.26933189821618</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>0.6639548655403902</v>
@@ -1259,7 +1259,7 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>0.07017635764339759</v>
+        <v>0.07017635819976679</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
@@ -1294,10 +1294,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>51.63017684017526</v>
+        <v>51.63017687344052</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>28.26579695102428</v>
+        <v>28.26579698882282</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>0.5053244878320772</v>
@@ -1312,7 +1312,7 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>-0.6345949737597965</v>
+        <v>-0.634594973815424</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
@@ -1347,10 +1347,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>71.14387143480535</v>
+        <v>71.14387138057266</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>36.11969027829939</v>
+        <v>36.11969026283181</v>
       </c>
       <c r="J17" s="2" t="n">
         <v>0.4134116033172695</v>
@@ -1365,7 +1365,7 @@
         <v>-1</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>0.1645810011723649</v>
+        <v>0.1645810012391424</v>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
@@ -1400,10 +1400,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>53.23083455005789</v>
+        <v>53.23083461253161</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>22.9516400415005</v>
+        <v>22.95164004150051</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>0.5460843204995706</v>
@@ -1418,7 +1418,7 @@
         <v>-1</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>-0.3531246933425762</v>
+        <v>-0.3531246934315972</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
@@ -1456,7 +1456,7 @@
         <v>51.93921035606791</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>23.12381053684191</v>
+        <v>23.12381055434743</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>0.7842704691768611</v>
@@ -1471,7 +1471,7 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>0.0027103237888756</v>
+        <v>0.0027103238000055</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
@@ -1506,10 +1506,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>44.40915747510478</v>
+        <v>44.40915745514376</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>15.14464573862796</v>
+        <v>15.14464573332165</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>0.2270158080671501</v>
@@ -1524,7 +1524,7 @@
         <v>-1</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>-0.0742537835436735</v>
+        <v>-0.0742537834991648</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
@@ -1559,10 +1559,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>60.70055988039058</v>
+        <v>60.70055989509937</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>41.10032647486013</v>
+        <v>41.10032645734289</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>1.013911217114202</v>
@@ -1577,7 +1577,7 @@
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>0.0752580332551296</v>
+        <v>0.075258033252905</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
@@ -1615,7 +1615,7 @@
         <v>54.08287236493935</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>15.87081657321302</v>
+        <v>15.87081671068779</v>
       </c>
       <c r="J22" s="2" t="n">
         <v>0.407092049387347</v>
@@ -1665,10 +1665,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>56.79220558377262</v>
+        <v>56.79220563949485</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>15.71171701028789</v>
+        <v>15.71171699557782</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>1.105566558177927</v>
@@ -1683,7 +1683,7 @@
         <v>-1</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>0.0256783707207232</v>
+        <v>0.0256783706873435</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
@@ -1718,10 +1718,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>53.48114735305222</v>
+        <v>53.48114741638003</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>27.67049570260034</v>
+        <v>27.67049570260033</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>0.6537112824940586</v>
@@ -1736,7 +1736,7 @@
         <v>-1</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>-0.0210725773454489</v>
+        <v>-0.0210725773565741</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
@@ -1771,7 +1771,7 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>55.48243570517651</v>
+        <v>55.48243583662349</v>
       </c>
       <c r="I25" s="2" t="n">
         <v>28.35361368408314</v>
@@ -1789,7 +1789,7 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>0.0247344406259506</v>
+        <v>0.0247344406281759</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
@@ -1810,7 +1810,7 @@
         <v/>
       </c>
       <c r="D26" s="2" t="n">
-        <v>496.2549857292479</v>
+        <v>496.2549857292478</v>
       </c>
       <c r="E26" s="2" t="n">
         <v>30.9</v>
@@ -1824,10 +1824,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>58.45887262375558</v>
+        <v>58.45887266453194</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>18.71366386828052</v>
+        <v>18.713663837435</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>0.7051406157625537</v>
@@ -1842,7 +1842,7 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>0.2561221695984589</v>
+        <v>0.2561221695762053</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
@@ -1877,10 +1877,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>48.82640971135586</v>
+        <v>48.82640981216053</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>12.2744445123444</v>
+        <v>12.2744445331203</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>1.531400252959722</v>
@@ -1930,10 +1930,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>49.6890941959791</v>
+        <v>49.68909399118995</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>21.08901632706459</v>
+        <v>21.08901630232535</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>0.7878205253041712</v>
@@ -1948,7 +1948,7 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>0.0164448750413579</v>
+        <v>0.0164448750747391</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
@@ -1983,10 +1983,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>42.50966776336448</v>
+        <v>42.50966780455239</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>28.89237810026683</v>
+        <v>28.89237817161342</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>2.508345645706944</v>
@@ -2036,10 +2036,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>39.6499231005707</v>
+        <v>39.64992306979794</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>20.79792211131302</v>
+        <v>20.7979221474125</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>0.5862350659408259</v>
@@ -2089,10 +2089,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46.10594747465212</v>
+        <v>46.10594746760585</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>17.46624585831511</v>
+        <v>17.46624590813425</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>0.4436552810998709</v>
@@ -2107,7 +2107,7 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>0.1259237993221172</v>
+        <v>0.1259237993443784</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
@@ -2145,7 +2145,7 @@
         <v>53.5877446750235</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>34.09691412721011</v>
+        <v>34.09691413495643</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>1.795983580426009</v>
@@ -2195,10 +2195,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>44.18436452915455</v>
+        <v>44.18436421506431</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>13.92977540369517</v>
+        <v>13.92977588778416</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>1.053801751042616</v>
@@ -2213,7 +2213,7 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>-0.0102843299819899</v>
+        <v>-0.0102843299466756</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
@@ -2248,10 +2248,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>36.43831637129214</v>
+        <v>36.43831643053608</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>21.99582910455362</v>
+        <v>21.9958290371751</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>2.528985684292139</v>
@@ -2301,10 +2301,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>37.29775226429642</v>
+        <v>37.29775221028437</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>27.13297719712186</v>
+        <v>27.13297722825114</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>0.6178356628006788</v>
@@ -2319,7 +2319,7 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>0.3779994407752971</v>
+        <v>0.377999440552772</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
@@ -2340,7 +2340,7 @@
         <v/>
       </c>
       <c r="D36" s="2" t="n">
-        <v>450.3570762676169</v>
+        <v>450.3570762676171</v>
       </c>
       <c r="E36" s="2" t="n">
         <v>74.5</v>
@@ -2354,10 +2354,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>43.20257747606914</v>
+        <v>43.20257743307304</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>8.542082375698199</v>
+        <v>8.542082409251947</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>0.5435439067548555</v>
@@ -2372,7 +2372,7 @@
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>-0.0541424027859738</v>
+        <v>-0.0541424028304857</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
@@ -2407,10 +2407,10 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>49.42826941589242</v>
+        <v>49.42826943641698</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>13.55143722092805</v>
+        <v>13.55143726049205</v>
       </c>
       <c r="J37" s="2" t="n">
         <v>0.5977734942476089</v>
@@ -2425,7 +2425,7 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>-0.0857500968731737</v>
+        <v>-0.0857500968843012</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
@@ -2460,7 +2460,7 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>54.70469487406808</v>
+        <v>54.70469492748363</v>
       </c>
       <c r="I38" s="2" t="n">
         <v>22.3018726441397</v>
@@ -2513,10 +2513,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>44.72683610069753</v>
+        <v>44.72683614761517</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>18.44940280019104</v>
+        <v>18.4494026846607</v>
       </c>
       <c r="J39" s="2" t="n">
         <v>0.7415643761119077</v>
@@ -2531,7 +2531,7 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>-0.1122256822793139</v>
+        <v>-0.1122256822904404</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
@@ -2566,10 +2566,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>57.08322822726369</v>
+        <v>57.08322830207274</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>17.18057368936899</v>
+        <v>17.18057358761949</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>1.201204532330209</v>
@@ -2584,7 +2584,7 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>0.0574064352045982</v>
+        <v>0.0574064351712171</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
@@ -2622,7 +2622,7 @@
         <v>50.7310841029356</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>12.38310167198658</v>
+        <v>12.38310163212458</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>0.7146941047175062</v>
@@ -2637,7 +2637,7 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>0.0077391385755187</v>
+        <v>0.0077391385710682</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
@@ -2672,10 +2672,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>55.02449391742635</v>
+        <v>55.02449396044642</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>23.67688712688496</v>
+        <v>23.67688712488708</v>
       </c>
       <c r="J42" s="2" t="n">
         <v>0.9556686811682706</v>
@@ -2690,7 +2690,7 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>0.09503921675873719</v>
+        <v>0.0950392167253578</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
@@ -2725,10 +2725,10 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>23.48532301472335</v>
+        <v>23.48532286123746</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>55.30601215380953</v>
+        <v>55.30601226880396</v>
       </c>
       <c r="J43" s="2" t="n">
         <v>0.7419841596453609</v>
@@ -2743,7 +2743,7 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>0.0029094900312419</v>
+        <v>0.0029094900534947</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
@@ -2764,7 +2764,7 @@
         <v/>
       </c>
       <c r="D44" s="2" t="n">
-        <v>393.1758889026943</v>
+        <v>393.1758889026947</v>
       </c>
       <c r="E44" s="2" t="n">
         <v>19.5</v>
@@ -2781,7 +2781,7 @@
         <v>35.01010917200365</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>25.93105855792507</v>
+        <v>25.93105855792506</v>
       </c>
       <c r="J44" s="2" t="n">
         <v>2.633623604883756</v>
@@ -2796,7 +2796,7 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>-0.0464793444631961</v>
+        <v>-0.0464793444854534</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
@@ -2831,10 +2831,10 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>49.18804503133477</v>
+        <v>49.18804492494377</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>12.27872909353246</v>
+        <v>12.27872914352922</v>
       </c>
       <c r="J45" s="2" t="n">
         <v>0.4851515203636359</v>
@@ -2849,7 +2849,7 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>0.0730598204930125</v>
+        <v>0.0730598205820274</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
@@ -2884,10 +2884,10 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>50.92365550605701</v>
+        <v>50.9236547500019</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>9.806276713361891</v>
+        <v>9.80627596338382</v>
       </c>
       <c r="J46" s="2" t="n">
         <v>0.0747420465119755</v>
@@ -2902,7 +2902,7 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>0.09611460400455581</v>
+        <v>0.09611460856668</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
@@ -2937,10 +2937,10 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>49.76664279490457</v>
+        <v>49.7666429023317</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>15.48193259133164</v>
+        <v>15.48193259426007</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>0.5075576072771187</v>
@@ -2955,7 +2955,7 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>-0.0126520573069006</v>
+        <v>-0.0126520573291546</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
@@ -2990,7 +2990,7 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>52.30168129203528</v>
+        <v>52.30168131835046</v>
       </c>
       <c r="I48" s="2" t="n">
         <v>27.20162805373186</v>
@@ -3043,10 +3043,10 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>48.27071856087006</v>
+        <v>48.27071877462282</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>11.9693411348231</v>
+        <v>11.96934108697152</v>
       </c>
       <c r="J49" s="2" t="n">
         <v>0.8735184449598299</v>
@@ -3061,7 +3061,7 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>0.0113185601657682</v>
+        <v>0.0113185601546401</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
@@ -3096,10 +3096,10 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>52.1648936802383</v>
+        <v>52.16489369128615</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>10.57232564303941</v>
+        <v>10.57232564408768</v>
       </c>
       <c r="J50" s="2" t="n">
         <v>0.3884383752219517</v>
@@ -3114,7 +3114,7 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>1.714778827295699</v>
+        <v>1.714778827095411</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
@@ -3149,7 +3149,7 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>46.5887190325304</v>
+        <v>46.58871902185003</v>
       </c>
       <c r="I51" s="2" t="n">
         <v>24.97273187999811</v>
@@ -3167,7 +3167,7 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>-0.0370862846289644</v>
+        <v>-0.0370862846245132</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
@@ -3202,10 +3202,10 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>50.73631477243313</v>
+        <v>50.73631478657666</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>8.566707797494177</v>
+        <v>8.566707766651756</v>
       </c>
       <c r="J52" s="2" t="n">
         <v>0.6607899626004681</v>
@@ -3220,7 +3220,7 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>-0.0144298796478403</v>
+        <v>-0.0144298796367095</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
@@ -3241,7 +3241,7 @@
         <v/>
       </c>
       <c r="D53" s="2" t="n">
-        <v>352.4093822999625</v>
+        <v>352.4093822999626</v>
       </c>
       <c r="E53" s="2" t="n">
         <v>7.11</v>
@@ -3255,10 +3255,10 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>50.93823418234832</v>
+        <v>50.93823418011675</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>10.20390864370355</v>
+        <v>10.2039087465847</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>0.1952270638936701</v>
@@ -3273,7 +3273,7 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>0.0675868625265706</v>
+        <v>0.0675868625376977</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
@@ -3308,10 +3308,10 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>30.33335353473473</v>
+        <v>30.33335354968206</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>24.70963798295186</v>
+        <v>24.70963799561322</v>
       </c>
       <c r="J54" s="2" t="n">
         <v>0</v>
@@ -3361,10 +3361,10 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>42.42273710004807</v>
+        <v>42.42273716006804</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>9.035857335734343</v>
+        <v>9.035857357254471</v>
       </c>
       <c r="J55" s="2" t="n">
         <v>0.3483373997759351</v>
@@ -3379,7 +3379,7 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>-0.0293021761028913</v>
+        <v>-0.0293021761473972</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
@@ -3400,7 +3400,7 @@
         <v/>
       </c>
       <c r="D56" s="2" t="n">
-        <v>344.4726968174039</v>
+        <v>344.4726968174029</v>
       </c>
       <c r="E56" s="2" t="n">
         <v>105.5</v>
@@ -3414,10 +3414,10 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>41.22010908431373</v>
+        <v>41.22010905508024</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>14.01687644298336</v>
+        <v>14.01687649796679</v>
       </c>
       <c r="J56" s="2" t="n">
         <v>1.67872921694417</v>
@@ -3432,7 +3432,7 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>-0.3796153903959114</v>
+        <v>-0.3796153901733557</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
@@ -3467,10 +3467,10 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>48.48313183366961</v>
+        <v>48.4831316874271</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>26.19789054601214</v>
+        <v>26.19789063435394</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>0.3359423949778098</v>
@@ -3485,7 +3485,7 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>0.0650936252673958</v>
+        <v>0.0650936253230323</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
@@ -3520,10 +3520,10 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>28.35692071737463</v>
+        <v>28.35692068898176</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>27.44815135022232</v>
+        <v>27.44815147606382</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>1.653008422598548</v>
@@ -3559,7 +3559,7 @@
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>337.5014318014991</v>
+        <v>337.5014318015</v>
       </c>
       <c r="E59" s="2" t="n">
         <v>26</v>
@@ -3573,10 +3573,10 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>38.63179023705977</v>
+        <v>38.63179017613456</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>27.71108267960776</v>
+        <v>27.71108271913661</v>
       </c>
       <c r="J59" s="2" t="n">
         <v>0.6761643598881846</v>
@@ -3591,7 +3591,7 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>-0.002391576385721</v>
+        <v>-0.0023915763523414</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
@@ -3612,7 +3612,7 @@
         <v/>
       </c>
       <c r="D60" s="2" t="n">
-        <v>337.3024659744194</v>
+        <v>337.3024659744196</v>
       </c>
       <c r="E60" s="2" t="n">
         <v>15.45</v>
@@ -3626,10 +3626,10 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>39.62140690004976</v>
+        <v>39.62140688176712</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>32.55773091442138</v>
+        <v>32.55773091961071</v>
       </c>
       <c r="J60" s="2" t="n">
         <v>0.5852551952054829</v>
@@ -3644,7 +3644,7 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>0.07935765030684699</v>
+        <v>0.07935765031797359</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
@@ -3665,7 +3665,7 @@
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>334.2416530707877</v>
+        <v>334.2416530707878</v>
       </c>
       <c r="E61" s="2" t="n">
         <v>32.65</v>
@@ -3679,10 +3679,10 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>50.76748480707426</v>
+        <v>50.76748506969586</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>8.232681516660033</v>
+        <v>8.232681467949597</v>
       </c>
       <c r="J61" s="2" t="n">
         <v>0.7607929230308067</v>
@@ -3697,7 +3697,7 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>0.0384647182931859</v>
+        <v>0.0384647181819148</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
@@ -3732,10 +3732,10 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>24.76761654329372</v>
+        <v>24.7676165751141</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>24.9465641585789</v>
+        <v>24.94656416567871</v>
       </c>
       <c r="J62" s="2" t="n">
         <v>3.092441738586137</v>
@@ -3750,7 +3750,7 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>-0.1118197576025184</v>
+        <v>-0.1118197575913933</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
@@ -3785,10 +3785,10 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>32.41645746766615</v>
+        <v>32.41645751337705</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>19.27713964822369</v>
+        <v>19.27713965175261</v>
       </c>
       <c r="J63" s="2" t="n">
         <v>0.951770542148195</v>
@@ -3803,7 +3803,7 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>-0.2440892928555463</v>
+        <v>-0.2440892929890712</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
@@ -3838,10 +3838,10 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>39.89126324080706</v>
+        <v>39.89126313163326</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>16.13051195168057</v>
+        <v>16.13051199636772</v>
       </c>
       <c r="J64" s="2" t="n">
         <v>0.7020971486000142</v>
@@ -3856,7 +3856,7 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>-0.1374133380681245</v>
+        <v>-0.1374133378789614</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
@@ -3877,7 +3877,7 @@
         <v/>
       </c>
       <c r="D65" s="2" t="n">
-        <v>322.1183274563284</v>
+        <v>322.1183274563285</v>
       </c>
       <c r="E65" s="2" t="n">
         <v>68.5</v>
@@ -3891,10 +3891,10 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>43.23004444130681</v>
+        <v>43.2300446207012</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>15.93433192821562</v>
+        <v>15.93433202775706</v>
       </c>
       <c r="J65" s="2" t="n">
         <v>0.7089900705847003</v>
@@ -3909,7 +3909,7 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>-0.3721517101080017</v>
+        <v>-0.372151710375047</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
@@ -3944,10 +3944,10 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>44.62162323283446</v>
+        <v>44.62162327761597</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>21.31044175539902</v>
+        <v>21.31044177157621</v>
       </c>
       <c r="J66" s="2" t="n">
         <v>0.5345146938859737</v>
@@ -3962,7 +3962,7 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>-0.0544585818943868</v>
+        <v>-0.0544585819388959</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
@@ -3983,7 +3983,7 @@
         <v/>
       </c>
       <c r="D67" s="2" t="n">
-        <v>320.9136727001994</v>
+        <v>320.9136727002009</v>
       </c>
       <c r="E67" s="2" t="n">
         <v>12.3</v>
@@ -3997,10 +3997,10 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>44.31604735532043</v>
+        <v>44.3160394761975</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>22.81993943831284</v>
+        <v>22.81993927290189</v>
       </c>
       <c r="J67" s="2" t="n">
         <v>0.4719151337708807</v>
@@ -4015,7 +4015,7 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>0.0012891706281601</v>
+        <v>0.0012891739106651</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
@@ -4050,10 +4050,10 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>43.16358200312141</v>
+        <v>43.16358167791867</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>10.65137082042527</v>
+        <v>10.65137093722135</v>
       </c>
       <c r="J68" s="2" t="n">
         <v>0.8809447083253089</v>
@@ -4068,7 +4068,7 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>-0.0169469592001902</v>
+        <v>-0.0169469590221569</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
@@ -4089,7 +4089,7 @@
         <v/>
       </c>
       <c r="D69" s="2" t="n">
-        <v>310.4276352766508</v>
+        <v>310.427635276651</v>
       </c>
       <c r="E69" s="2" t="n">
         <v>17.1</v>
@@ -4103,10 +4103,10 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>43.29169746622856</v>
+        <v>43.29169752996959</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>18.6388506235312</v>
+        <v>18.63885062505226</v>
       </c>
       <c r="J69" s="2" t="n">
         <v>0.911360284080754</v>
@@ -4156,10 +4156,10 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>43.14906615127083</v>
+        <v>43.14906605106527</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>23.50223988705314</v>
+        <v>23.50224000727427</v>
       </c>
       <c r="J70" s="2" t="n">
         <v>0.5120523351121652</v>
@@ -4174,7 +4174,7 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>0.1264880517141436</v>
+        <v>0.1264880517809049</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
@@ -4209,10 +4209,10 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>44.43546668675432</v>
+        <v>44.4354667579651</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>18.87600789052682</v>
+        <v>18.87600785958044</v>
       </c>
       <c r="J71" s="2" t="n">
         <v>0.1499276599040962</v>
@@ -4227,7 +4227,7 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>-0.1577845764281358</v>
+        <v>-0.1577845764837742</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
@@ -4248,7 +4248,7 @@
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>297.8901220404103</v>
+        <v>297.8901220404102</v>
       </c>
       <c r="E72" s="2" t="n">
         <v>13.05</v>
@@ -4262,10 +4262,10 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>44.63866022279278</v>
+        <v>44.63866026332624</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>20.77728980728407</v>
+        <v>20.77728986345522</v>
       </c>
       <c r="J72" s="2" t="n">
         <v>0.502963476140964</v>
@@ -4315,10 +4315,10 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>51.5678248157296</v>
+        <v>51.56782484695619</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>12.99633628037481</v>
+        <v>12.99633626789948</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>1.603768348902477</v>
@@ -4333,7 +4333,7 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>-0.0309995603814466</v>
+        <v>-0.0309995603703189</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
@@ -4354,7 +4354,7 @@
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>292.9792414255561</v>
+        <v>292.9792414255554</v>
       </c>
       <c r="E74" s="2" t="n">
         <v>699</v>
@@ -4371,7 +4371,7 @@
         <v>44.12876814630479</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>11.31046961010666</v>
+        <v>11.31046964208165</v>
       </c>
       <c r="J74" s="2" t="n">
         <v>0.4262569204174543</v>
@@ -4386,7 +4386,7 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>-2.325496132454834</v>
+        <v>-2.325496131564828</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
@@ -4407,7 +4407,7 @@
         <v/>
       </c>
       <c r="D75" s="2" t="n">
-        <v>292.2727637231951</v>
+        <v>292.2727637231952</v>
       </c>
       <c r="E75" s="2" t="n">
         <v>276.5</v>
@@ -4421,10 +4421,10 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>27.6006514368144</v>
+        <v>27.6006512046645</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>39.59134505989268</v>
+        <v>39.59134512526497</v>
       </c>
       <c r="J75" s="2" t="n">
         <v>1.101667727907232</v>
@@ -4439,7 +4439,7 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>-0.7220464013706298</v>
+        <v>-0.7220463999241034</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
@@ -4474,10 +4474,10 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>39.69797596997519</v>
+        <v>39.6979772051025</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>22.84733814630626</v>
+        <v>22.84733844636558</v>
       </c>
       <c r="J76" s="2" t="n">
         <v>0.4376298873520786</v>
@@ -4492,7 +4492,7 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>0.009058500241062599</v>
+        <v>0.009058499985138401</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
@@ -4527,10 +4527,10 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>48.14675887273457</v>
+        <v>48.14675865393064</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>22.71983757968933</v>
+        <v>22.71983768833963</v>
       </c>
       <c r="J77" s="2" t="n">
         <v>0.5794892233667036</v>
@@ -4545,7 +4545,7 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>0.1215759979187395</v>
+        <v>0.1215759980633953</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
@@ -4583,7 +4583,7 @@
         <v>51.21739120090434</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>11.48208651725725</v>
+        <v>11.4820865086376</v>
       </c>
       <c r="J78" s="2" t="n">
         <v>1.508667725671662</v>
@@ -4633,10 +4633,10 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>36.72531320496911</v>
+        <v>36.72531310545264</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>37.98356660496544</v>
+        <v>37.9835667983133</v>
       </c>
       <c r="J79" s="2" t="n">
         <v>0.7091782403611994</v>
@@ -4651,7 +4651,7 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>0.3264349120216505</v>
+        <v>0.3264349122441907</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
@@ -4686,10 +4686,10 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>42.71665586666957</v>
+        <v>42.71665582985549</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>9.140662893558956</v>
+        <v>9.140662916425883</v>
       </c>
       <c r="J80" s="2" t="n">
         <v>0.918806715129435</v>
@@ -4704,7 +4704,7 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>-0.0378001681185071</v>
+        <v>-0.0378001679849754</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
@@ -4739,10 +4739,10 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>50.21515326515548</v>
+        <v>50.2151533295398</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>12.34245617887821</v>
+        <v>12.34245620786279</v>
       </c>
       <c r="J81" s="2" t="n">
         <v>0.4095651925805789</v>
@@ -4792,10 +4792,10 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>45.35370215381646</v>
+        <v>45.35370189206611</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>16.77278616033155</v>
+        <v>16.77278629394617</v>
       </c>
       <c r="J82" s="2" t="n">
         <v>0.4670247023880471</v>
@@ -4810,7 +4810,7 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>-0.2187264451033156</v>
+        <v>-0.2187264446582409</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
@@ -4831,7 +4831,7 @@
         <v/>
       </c>
       <c r="D83" s="2" t="n">
-        <v>255.2791340115592</v>
+        <v>255.2791340115593</v>
       </c>
       <c r="E83" s="2" t="n">
         <v>6.25</v>
@@ -4845,10 +4845,10 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>31.90709043628356</v>
+        <v>31.90709045807145</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>22.6108859698442</v>
+        <v>22.610885998567</v>
       </c>
       <c r="J83" s="2" t="n">
         <v>1.267694664083302</v>
@@ -4863,7 +4863,7 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>-0.010936478126146</v>
+        <v>-0.0109364781328225</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
@@ -4884,7 +4884,7 @@
         <v/>
       </c>
       <c r="D84" s="2" t="n">
-        <v>255.2454065857505</v>
+        <v>255.2454065857506</v>
       </c>
       <c r="E84" s="2" t="n">
         <v>17.45</v>
@@ -4898,10 +4898,10 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>40.38847264881744</v>
+        <v>40.38847240937753</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>32.06027476096221</v>
+        <v>32.06027486959128</v>
       </c>
       <c r="J84" s="2" t="n">
         <v>0.6225557950428553</v>
@@ -4916,7 +4916,7 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>-0.0039314140558742</v>
+        <v>-0.0039314138842467</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
@@ -4937,7 +4937,7 @@
         <v/>
       </c>
       <c r="D85" s="2" t="n">
-        <v>251.6014864706743</v>
+        <v>251.6014864706753</v>
       </c>
       <c r="E85" s="2" t="n">
         <v>66</v>
@@ -4951,10 +4951,10 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>48.37591118037257</v>
+        <v>48.37591114242193</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>12.05625701010428</v>
+        <v>12.05625710173019</v>
       </c>
       <c r="J85" s="2" t="n">
         <v>0.2763589828495598</v>
@@ -4969,7 +4969,7 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>-0.125174743737088</v>
+        <v>-0.1251747436703258</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
@@ -5004,10 +5004,10 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>39.6541399191126</v>
+        <v>39.65414005025227</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>7.558030916863396</v>
+        <v>7.558030902244351</v>
       </c>
       <c r="J86" s="2" t="n">
         <v>2.986749443468509</v>
@@ -5022,7 +5022,7 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>0.0146174883849338</v>
+        <v>0.0146174883292986</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
@@ -5060,7 +5060,7 @@
         <v>33.06635877516952</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>23.33689467604703</v>
+        <v>23.33689468688239</v>
       </c>
       <c r="J87" s="2" t="n">
         <v>0.4179182929817769</v>
@@ -5110,10 +5110,10 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>48.71433743579543</v>
+        <v>48.71433746003079</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>5.930345847115438</v>
+        <v>5.930345877287301</v>
       </c>
       <c r="J88" s="2" t="n">
         <v>0.436274081950618</v>
@@ -5128,7 +5128,7 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>0.0415502904453151</v>
+        <v>0.0415502904341879</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
@@ -5166,7 +5166,7 @@
         <v>43.88170428445039</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>15.08183058431626</v>
+        <v>15.08183060356054</v>
       </c>
       <c r="J89" s="2" t="n">
         <v>0.5186073575128568</v>
@@ -5181,7 +5181,7 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>0.0155526809358521</v>
+        <v>0.0155526809447538</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
@@ -5216,10 +5216,10 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>42.16577189361502</v>
+        <v>42.16577188899697</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>10.29497635124557</v>
+        <v>10.29497638536218</v>
       </c>
       <c r="J90" s="2" t="n">
         <v>0.168613957688645</v>
@@ -5234,7 +5234,7 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>0.0310783092013129</v>
+        <v>0.0310783091946367</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
@@ -5269,10 +5269,10 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>49.16387774062459</v>
+        <v>49.16387776089812</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>14.44930207460586</v>
+        <v>14.44930207468676</v>
       </c>
       <c r="J91" s="2" t="n">
         <v>1.351277911539894</v>
@@ -5322,10 +5322,10 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>34.03165134729996</v>
+        <v>34.03165139728567</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>24.15595550882902</v>
+        <v>24.15595555901442</v>
       </c>
       <c r="J92" s="2" t="n">
         <v>0.2697946046931946</v>
@@ -5340,7 +5340,7 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>-0.0216342541357427</v>
+        <v>-0.021634254146869</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
@@ -5375,7 +5375,7 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>32.59704687693366</v>
+        <v>32.59704685672858</v>
       </c>
       <c r="I93" s="2" t="n">
         <v>29.78140838246116</v>
@@ -5428,10 +5428,10 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>46.59781347622856</v>
+        <v>46.59781340263403</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>14.5512646240608</v>
+        <v>14.55126467028614</v>
       </c>
       <c r="J94" s="2" t="n">
         <v>0.5180395055277867</v>
@@ -5446,7 +5446,7 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>-0.241526160709038</v>
+        <v>-0.2415261605977617</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
@@ -5481,10 +5481,10 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>43.75689456264242</v>
+        <v>43.7568946610978</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>14.52606955811724</v>
+        <v>14.52606964115181</v>
       </c>
       <c r="J95" s="2" t="n">
         <v>1.061136792964763</v>
@@ -5499,7 +5499,7 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>-0.0083989865191862</v>
+        <v>-0.0083989865303126</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
@@ -5534,10 +5534,10 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>48.6457856648475</v>
+        <v>48.64578571277686</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>12.18296464062828</v>
+        <v>12.18296468119942</v>
       </c>
       <c r="J96" s="2" t="n">
         <v>0.2249250096795675</v>
@@ -5552,7 +5552,7 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>-0.08381279588639851</v>
+        <v>-0.08381279595315751</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
@@ -5587,10 +5587,10 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>33.17979786824418</v>
+        <v>33.17979777692447</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>8.769809602556821</v>
+        <v>8.769809536284505</v>
       </c>
       <c r="J97" s="2" t="n">
         <v>0.7535309221377681</v>
@@ -5605,7 +5605,7 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>-0.4561794846315825</v>
+        <v>-0.4561794838526847</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
@@ -5640,10 +5640,10 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>40.61848534278261</v>
+        <v>40.61848539298406</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>17.86580193502385</v>
+        <v>17.86580194258671</v>
       </c>
       <c r="J98" s="2" t="n">
         <v>0.4362253128082805</v>
@@ -5658,7 +5658,7 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>0.0126355083886178</v>
+        <v>0.0126355083663625</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
@@ -5696,7 +5696,7 @@
         <v>50.91200446564194</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>8.92065751425168</v>
+        <v>8.92065743071935</v>
       </c>
       <c r="J99" s="2" t="n">
         <v>0.603459583538285</v>
@@ -5711,7 +5711,7 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>0.3059918046846929</v>
+        <v>0.3059918036975808</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
@@ -5746,10 +5746,10 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>34.86046120086584</v>
+        <v>34.8604613306469</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>32.47825076977574</v>
+        <v>32.47825078960295</v>
       </c>
       <c r="J100" s="2" t="n">
         <v>0.7728841266485443</v>
@@ -5764,7 +5764,7 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>0.002911906848098</v>
+        <v>0.0029119068035889</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
@@ -5802,7 +5802,7 @@
         <v>41.08444409117836</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>10.97575308408577</v>
+        <v>10.97575311375755</v>
       </c>
       <c r="J101" s="2" t="n">
         <v>0.8187801994017417</v>
@@ -5817,7 +5817,7 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>0.0050552602111418</v>
+        <v>0.0050552602222698</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
@@ -5852,7 +5852,7 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>39.5403746782918</v>
+        <v>39.5403746354615</v>
       </c>
       <c r="I102" s="2" t="n">
         <v>23.16158012845588</v>
@@ -5870,7 +5870,7 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>-0.0581086230829653</v>
+        <v>-0.0581086232164911</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
@@ -5891,7 +5891,7 @@
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>210.8729195606531</v>
+        <v>210.8729195606529</v>
       </c>
       <c r="E103" s="2" t="n">
         <v>23.05</v>
@@ -5905,10 +5905,10 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>45.25963943182494</v>
+        <v>45.25963941071828</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>5.119036154578149</v>
+        <v>5.119036158802952</v>
       </c>
       <c r="J103" s="2" t="n">
         <v>0.8622069614414106</v>
@@ -5923,7 +5923,7 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>-0.0033726784687696</v>
+        <v>-0.0033726784242615</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
@@ -5958,10 +5958,10 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>50.43547673679654</v>
+        <v>50.43547668344164</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>18.06665908503258</v>
+        <v>18.06665903120349</v>
       </c>
       <c r="J104" s="2" t="n">
         <v>0.9288049767465556</v>
@@ -5997,7 +5997,7 @@
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>194.2179619016106</v>
+        <v>194.2179619016094</v>
       </c>
       <c r="E105" s="2" t="n">
         <v>64.40000000000001</v>
@@ -6011,7 +6011,7 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>51.18018451381249</v>
+        <v>51.1801845104879</v>
       </c>
       <c r="I105" s="2" t="n">
         <v>21.542490833729</v>
@@ -6029,7 +6029,7 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>-1.184543157539203</v>
+        <v>-1.184543157516954</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
@@ -6064,10 +6064,10 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>42.75937508015001</v>
+        <v>42.75937494302369</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>16.36644321871258</v>
+        <v>16.36644328919786</v>
       </c>
       <c r="J106" s="2" t="n">
         <v>1.081609927212568</v>
@@ -6082,7 +6082,7 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>0.0069930215937528</v>
+        <v>0.0069930216382601</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
@@ -6117,10 +6117,10 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>45.46547030186201</v>
+        <v>45.46547029883565</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>13.19563541064757</v>
+        <v>13.19563546358064</v>
       </c>
       <c r="J107" s="2" t="n">
         <v>0.5325164438786336</v>
@@ -6156,7 +6156,7 @@
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>177.8432355317164</v>
+        <v>177.8432355317171</v>
       </c>
       <c r="E108" s="2" t="n">
         <v>196</v>
@@ -6170,10 +6170,10 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>43.30531215740378</v>
+        <v>43.3053121204459</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>10.00399064412504</v>
+        <v>10.00399061324159</v>
       </c>
       <c r="J108" s="2" t="n">
         <v>0.425144086768141</v>
@@ -6188,7 +6188,7 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>-0.54228181406623</v>
+        <v>-0.5422818135098741</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
@@ -6223,10 +6223,10 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>48.39437996819087</v>
+        <v>48.39437984241511</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>12.54145300237842</v>
+        <v>12.5414530121041</v>
       </c>
       <c r="J109" s="2" t="n">
         <v>0.5535224586928081</v>
@@ -6241,7 +6241,7 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>0.0512900796150477</v>
+        <v>0.051290079603922</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
@@ -6276,10 +6276,10 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>52.77989777541445</v>
+        <v>52.77989777384564</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>9.1671226089423</v>
+        <v>9.167122732721641</v>
       </c>
       <c r="J110" s="2" t="n">
         <v>0.4798771552722107</v>
@@ -6329,10 +6329,10 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>45.75353411473413</v>
+        <v>45.75353481040914</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>11.43605779883075</v>
+        <v>11.43605780109266</v>
       </c>
       <c r="J111" s="2" t="n">
         <v>0.0001400550416313</v>
@@ -6382,10 +6382,10 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>51.91879873819772</v>
+        <v>51.91879876999717</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>19.44384807457648</v>
+        <v>19.44384805724503</v>
       </c>
       <c r="J112" s="2" t="n">
         <v>0.2236906510034263</v>
@@ -6400,7 +6400,7 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>0.040437559178269</v>
+        <v>0.0404375591337598</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
@@ -6435,10 +6435,10 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>47.78896365929295</v>
+        <v>47.78896380223252</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>15.68770203533845</v>
+        <v>15.6877020822982</v>
       </c>
       <c r="J113" s="2" t="n">
         <v>1.138063168865906</v>
@@ -6453,7 +6453,7 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>0.0102298858998013</v>
+        <v>0.0102298857662753</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
@@ -6488,10 +6488,10 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>32.86232830231734</v>
+        <v>32.86232835427593</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>19.10831852076622</v>
+        <v>19.1083185270153</v>
       </c>
       <c r="J114" s="2" t="n">
         <v>0.3016058633221153</v>
@@ -6506,7 +6506,7 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>-0.1218205302602301</v>
+        <v>-0.1218205302713583</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
@@ -6541,10 +6541,10 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>49.90280756175169</v>
+        <v>49.9028075076608</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>12.69467972535677</v>
+        <v>12.69467974136995</v>
       </c>
       <c r="J115" s="2" t="n">
         <v>1.087615949355959</v>
@@ -6559,7 +6559,7 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-0.0005648758012771</v>
+        <v>-0.0005648757901528</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
@@ -6594,10 +6594,10 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>38.80466804510702</v>
+        <v>38.80466817390331</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>9.51976021130945</v>
+        <v>9.519760325191257</v>
       </c>
       <c r="J116" s="2" t="n">
         <v>0.9554569055577288</v>
@@ -6612,7 +6612,7 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>0.0102867785153978</v>
+        <v>0.0102867784909188</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
@@ -6647,10 +6647,10 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>41.02453300258299</v>
+        <v>41.02453308743376</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>10.16589351099681</v>
+        <v>10.16589345732232</v>
       </c>
       <c r="J117" s="2" t="n">
         <v>0.1011474815970939</v>
@@ -6665,7 +6665,7 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>-0.0017563047101163</v>
+        <v>-0.0017563047323714</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
@@ -6700,10 +6700,10 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>36.77541204876096</v>
+        <v>36.7754120780831</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>23.03727374614221</v>
+        <v>23.03727390729559</v>
       </c>
       <c r="J118" s="2" t="n">
         <v>0.1997971702293157</v>
@@ -6718,7 +6718,7 @@
         <v>-1</v>
       </c>
       <c r="N118" s="2" t="n">
-        <v>-0.0115572104211656</v>
+        <v>-0.0115572103766573</v>
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
@@ -6753,10 +6753,10 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>37.80698450167327</v>
+        <v>37.80698417416073</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>17.25404851467422</v>
+        <v>17.25404869356028</v>
       </c>
       <c r="J119" s="2" t="n">
         <v>0.09485171628344451</v>
@@ -6771,7 +6771,7 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>-0.0140613970190381</v>
+        <v>-0.0140613969411473</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
@@ -6806,10 +6806,10 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>39.10305957349571</v>
+        <v>39.10305949766703</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>15.84860774067127</v>
+        <v>15.84860767673352</v>
       </c>
       <c r="J120" s="2" t="n">
         <v>0.2898815301299903</v>
@@ -6824,7 +6824,7 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>0.06391953048078711</v>
+        <v>0.06391953056980711</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
@@ -6845,7 +6845,7 @@
         <v/>
       </c>
       <c r="D121" s="2" t="n">
-        <v>150.6907412260264</v>
+        <v>150.6907412260263</v>
       </c>
       <c r="E121" s="2" t="n">
         <v>79.59999999999999</v>
@@ -6859,10 +6859,10 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>41.33665306039034</v>
+        <v>41.33665354397382</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>10.76942234848532</v>
+        <v>10.76942273546453</v>
       </c>
       <c r="J121" s="2" t="n">
         <v>0.5036580712732786</v>
@@ -6877,7 +6877,7 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>0.1293157691710231</v>
+        <v>0.1293157696161082</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
@@ -6898,7 +6898,7 @@
         <v/>
       </c>
       <c r="D122" s="2" t="n">
-        <v>147.7983562297197</v>
+        <v>147.7983562297198</v>
       </c>
       <c r="E122" s="2" t="n">
         <v>9.19</v>
@@ -6912,10 +6912,10 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>46.17349648567914</v>
+        <v>46.17349666955876</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>8.802496472927102</v>
+        <v>8.802496467773832</v>
       </c>
       <c r="J122" s="2" t="n">
         <v>0.3445227478682101</v>
@@ -6930,7 +6930,7 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>0.005949713040227</v>
+        <v>0.0059497129957167</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
@@ -6951,7 +6951,7 @@
         <v/>
       </c>
       <c r="D123" s="2" t="n">
-        <v>143.2164431712961</v>
+        <v>143.216443171296</v>
       </c>
       <c r="E123" s="2" t="n">
         <v>14.35</v>
@@ -6965,10 +6965,10 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>47.14649688258773</v>
+        <v>47.14649684961105</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>11.92050045338421</v>
+        <v>11.92050058084785</v>
       </c>
       <c r="J123" s="2" t="n">
         <v>0.5152589055244483</v>
@@ -7018,10 +7018,10 @@
         <v>0</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>43.64610464171341</v>
+        <v>43.64610452882009</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>19.23217675365634</v>
+        <v>19.2321769938357</v>
       </c>
       <c r="J124" s="2" t="n">
         <v>0.1051216414652538</v>
@@ -7036,7 +7036,7 @@
         <v>-1</v>
       </c>
       <c r="N124" s="2" t="n">
-        <v>0.0159319405502945</v>
+        <v>0.0159319406615676</v>
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
@@ -7071,7 +7071,7 @@
         <v>0</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>36.18091053745876</v>
+        <v>36.18091049785818</v>
       </c>
       <c r="I125" s="2" t="n">
         <v>9.354981228073022</v>
@@ -7089,7 +7089,7 @@
         <v>-1</v>
       </c>
       <c r="N125" s="2" t="n">
-        <v>-0.0036221741302361</v>
+        <v>-0.0036221741079822</v>
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>
@@ -7127,7 +7127,7 @@
         <v>39.06292270622599</v>
       </c>
       <c r="I126" s="2" t="n">
-        <v>9.452739850796</v>
+        <v>9.452739850795997</v>
       </c>
       <c r="J126" s="2" t="n">
         <v>0.7371579717980277</v>
@@ -7142,7 +7142,7 @@
         <v>-1</v>
       </c>
       <c r="N126" s="2" t="n">
-        <v>-0.0005736163092595001</v>
+        <v>-0.000573616311485</v>
       </c>
       <c r="O126" s="2" t="inlineStr">
         <is>
@@ -7177,10 +7177,10 @@
         <v>0</v>
       </c>
       <c r="H127" s="2" t="n">
-        <v>50.927326741284</v>
+        <v>50.92732666269455</v>
       </c>
       <c r="I127" s="2" t="n">
-        <v>10.55419107618756</v>
+        <v>10.55419110475697</v>
       </c>
       <c r="J127" s="2" t="n">
         <v>0.7333678287830576</v>
@@ -7195,7 +7195,7 @@
         <v>-1</v>
       </c>
       <c r="N127" s="2" t="n">
-        <v>-0.0101972522932754</v>
+        <v>-0.0101972522821483</v>
       </c>
       <c r="O127" s="2" t="inlineStr">
         <is>
@@ -7230,10 +7230,10 @@
         <v>0</v>
       </c>
       <c r="H128" s="2" t="n">
-        <v>39.96116754927892</v>
+        <v>39.9611678999597</v>
       </c>
       <c r="I128" s="2" t="n">
-        <v>18.30873243307893</v>
+        <v>18.30873238528409</v>
       </c>
       <c r="J128" s="2" t="n">
         <v>0.5127334465195246</v>
@@ -7286,7 +7286,7 @@
         <v>41.89733806673743</v>
       </c>
       <c r="I129" s="2" t="n">
-        <v>14.10139034621174</v>
+        <v>14.10139043644395</v>
       </c>
       <c r="J129" s="2" t="n">
         <v>0.9779548285610944</v>
@@ -7301,7 +7301,7 @@
         <v>-1</v>
       </c>
       <c r="N129" s="2" t="n">
-        <v>-0.0484924270252753</v>
+        <v>-0.0484924269807692</v>
       </c>
       <c r="O129" s="2" t="inlineStr">
         <is>
@@ -7322,7 +7322,7 @@
         <v/>
       </c>
       <c r="D130" s="2" t="n">
-        <v>89.49831170708893</v>
+        <v>89.49831170708894</v>
       </c>
       <c r="E130" s="2" t="n">
         <v>45.6</v>
@@ -7339,7 +7339,7 @@
         <v>49.14989578507964</v>
       </c>
       <c r="I130" s="2" t="n">
-        <v>13.93374915212161</v>
+        <v>13.93374908496215</v>
       </c>
       <c r="J130" s="2" t="n">
         <v>0.7975212146144058</v>
@@ -7392,7 +7392,7 @@
         <v>42.81461527802914</v>
       </c>
       <c r="I131" s="2" t="n">
-        <v>15.55587129457165</v>
+        <v>15.55587131983602</v>
       </c>
       <c r="J131" s="2" t="n">
         <v>0.5619201813244366</v>
@@ -7442,10 +7442,10 @@
         <v>0</v>
       </c>
       <c r="H132" s="2" t="n">
-        <v>51.74505581842296</v>
+        <v>51.74505590915226</v>
       </c>
       <c r="I132" s="2" t="n">
-        <v>11.7786327326755</v>
+        <v>11.77863273267551</v>
       </c>
       <c r="J132" s="2" t="n">
         <v>0.6524428229882353</v>
@@ -7460,7 +7460,7 @@
         <v>-1</v>
       </c>
       <c r="N132" s="2" t="n">
-        <v>0.0160344867030118</v>
+        <v>0.0160344866918867</v>
       </c>
       <c r="O132" s="2" t="inlineStr">
         <is>
@@ -7498,7 +7498,7 @@
         <v>44.53314504609418</v>
       </c>
       <c r="I133" s="2" t="n">
-        <v>12.80569386850856</v>
+        <v>12.8056938969914</v>
       </c>
       <c r="J133" s="2" t="n">
         <v>0.2469258623831483</v>

</xml_diff>